<commit_message>
Give each night post its own caption
Night captions reused one text per month (12 texts for 364 days).
Each now cites the day's verse reference and rotates the call to action.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KvHsXRHqPeMpS6fZDvb3az
</commit_message>
<xml_diff>
--- a/legendas-365.xlsx
+++ b/legendas-365.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Salmos 36:7. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -578,7 +578,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Salmos 63:3. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
@@ -621,7 +621,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Cantares 8:7. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Gálatas 5:13-14. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -793,7 +793,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com João 15:9. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -836,7 +836,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Efésios 2:4-5. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
@@ -879,7 +879,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Romanos 12:9. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
@@ -922,7 +922,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Provérbios 10:12. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
@@ -965,7 +965,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com 1 João 4:20. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Salmos 86:15. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Oseias 11:4. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Marcos 10:21. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
@@ -1137,7 +1137,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com João 21:17. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Tito 3:4-5. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com 1 Coríntios 16:14. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Jeremias 33:3. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Mateus 7:7-8. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
@@ -1352,7 +1352,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com 1 Tessalonicenses 5:17. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Filipenses 4:19. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
@@ -1438,7 +1438,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Salmos 37:4. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Salmos 56:8. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
@@ -1524,7 +1524,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Marcos 11:24. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr"/>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Salmos 145:18. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Mateus 6:6. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr"/>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Romanos 8:26. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Hebreus 4:16. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr"/>
@@ -1739,7 +1739,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Salmos 62:8. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Tiago 5:16. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr"/>
@@ -1825,7 +1825,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Mateus 6:9-10. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
@@ -1868,7 +1868,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Salmos 5:3. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr"/>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Lucas 22:42. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr"/>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com 1 João 5:14. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr"/>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Salmos 20:7. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr"/>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Isaías 65:24. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr"/>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Neemias 1:4. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Daniel 9:18. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr"/>
@@ -2169,7 +2169,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Salmos 37:7. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr"/>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Mateus 21:22. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr"/>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Salmos 141:2. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Isaías 30:15. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr"/>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Salmos 9:10. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Atos 12:5. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr"/>
@@ -2427,7 +2427,7 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Lucas 11:9-10. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr"/>
@@ -2470,7 +2470,7 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Provérbios 29:25. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr"/>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: oração e confiança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #oracao</t>
+          <t>Oração da noite: oração e confiança 🌙 Para fechar o dia com Salmos 57:1-2. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #oracao</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr"/>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Isaías 43:18. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr"/>
@@ -2599,7 +2599,7 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Filipenses 3:13-14. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr"/>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Ezequiel 36:26. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr"/>
@@ -2685,7 +2685,7 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Apocalipse 21:5. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr"/>
@@ -2728,7 +2728,7 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Salmos 40:3. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr"/>
@@ -2771,7 +2771,7 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com 2 Coríntios 1:20. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr"/>
@@ -2814,7 +2814,7 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Números 23:19. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr"/>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Josué 21:45. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr"/>
@@ -2900,7 +2900,7 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Lamentações 3:25. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr"/>
@@ -2943,7 +2943,7 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Isaías 55:10-11. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr"/>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Salmos 37:25. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr"/>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Deuteronômio 7:9. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr"/>
@@ -3072,7 +3072,7 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Hebreus 10:23. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr"/>
@@ -3115,7 +3115,7 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Jonas 2:10. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr"/>
@@ -3158,7 +3158,7 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Jonas 3:1. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr"/>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Isaías 58:11. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr"/>
@@ -3244,7 +3244,7 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Salmos 23:6. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr"/>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Gênesis 28:15. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr"/>
@@ -3330,7 +3330,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Isaías 42:3. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr"/>
@@ -3373,7 +3373,7 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Salmos 145:14. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr"/>
@@ -3416,7 +3416,7 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Isaías 60:1. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr"/>
@@ -3459,7 +3459,7 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Atos 9:17-18. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr"/>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Lucas 5:5-6. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr"/>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Oseias 6:3. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr"/>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Ageu 2:9. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr"/>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Isaías 54:10. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr"/>
@@ -3674,7 +3674,7 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Salmos 30:11. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr"/>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com 2 Pedro 3:9. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr"/>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Isaías 46:4. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr"/>
@@ -3803,7 +3803,7 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Números 6:24-26. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr"/>
@@ -3846,7 +3846,7 @@
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: recomeço e promessas 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
+          <t>Oração da noite: recomeço e promessas 🌙 Para fechar o dia com Judas 1:24-25. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #recomeco</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr"/>
@@ -3889,7 +3889,7 @@
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Filipenses 4:6-7. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr"/>
@@ -3932,7 +3932,7 @@
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Mateus 6:34. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr"/>
@@ -3975,7 +3975,7 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com 1 Pedro 5:7. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr"/>
@@ -4018,7 +4018,7 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com João 14:27. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr"/>
@@ -4061,7 +4061,7 @@
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Salmos 94:19. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr"/>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Isaías 26:3. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr"/>
@@ -4147,7 +4147,7 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Salmos 46:10. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr"/>
@@ -4190,7 +4190,7 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Mateus 11:28-30. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr"/>
@@ -4233,7 +4233,7 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Salmos 55:22. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr"/>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Provérbios 12:25. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr"/>
@@ -4319,7 +4319,7 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Salmos 4:8. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr"/>
@@ -4362,7 +4362,7 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Isaías 41:10. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr"/>
@@ -4405,7 +4405,7 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Salmos 23:1-3. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr"/>
@@ -4448,7 +4448,7 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Romanos 8:28. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr"/>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com 2 Timóteo 1:7. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr"/>
@@ -4534,7 +4534,7 @@
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Salmos 34:4. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr"/>
@@ -4577,7 +4577,7 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Salmos 61:2. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr"/>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Filipenses 4:8. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr"/>
@@ -4663,7 +4663,7 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Salmos 139:23-24. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr"/>
@@ -4706,7 +4706,7 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Lucas 12:25-26. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr"/>
@@ -4749,7 +4749,7 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Josué 1:9. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr"/>
@@ -4792,7 +4792,7 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Salmos 121:1-2. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr"/>
@@ -4835,7 +4835,7 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Isaías 40:31. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr"/>
@@ -4878,7 +4878,7 @@
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Êxodo 14:14. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr"/>
@@ -4921,7 +4921,7 @@
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Salmos 56:3. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr"/>
@@ -4964,7 +4964,7 @@
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Mateus 6:26. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr"/>
@@ -5007,7 +5007,7 @@
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Salmos 3:3. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr"/>
@@ -5050,7 +5050,7 @@
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Sofonias 3:17. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I107" s="2" t="inlineStr"/>
@@ -5093,7 +5093,7 @@
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com João 16:33. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr"/>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Salmos 16:8. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I109" s="2" t="inlineStr"/>
@@ -5179,7 +5179,7 @@
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: ansiedade e paz 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #ansiedade</t>
+          <t>Oração da noite: ansiedade e paz 🌙 Para fechar o dia com Salmos 27:1. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #ansiedade</t>
         </is>
       </c>
       <c r="I110" s="2" t="inlineStr"/>
@@ -5222,7 +5222,7 @@
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Deuteronômio 31:6. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I111" s="2" t="inlineStr"/>
@@ -5265,7 +5265,7 @@
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Salmos 118:6. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I112" s="2" t="inlineStr"/>
@@ -5308,7 +5308,7 @@
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Isaías 43:1-2. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I113" s="2" t="inlineStr"/>
@@ -5351,7 +5351,7 @@
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Salmos 23:4. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr"/>
@@ -5394,7 +5394,7 @@
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Romanos 8:31. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I115" s="2" t="inlineStr"/>
@@ -5437,7 +5437,7 @@
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Hebreus 13:6. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I116" s="2" t="inlineStr"/>
@@ -5480,7 +5480,7 @@
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Provérbios 28:1. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I117" s="2" t="inlineStr"/>
@@ -5523,7 +5523,7 @@
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Salmos 91:1-2. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I118" s="2" t="inlineStr"/>
@@ -5566,7 +5566,7 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Josué 1:7. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I119" s="2" t="inlineStr"/>
@@ -5609,7 +5609,7 @@
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com 1 Samuel 17:45. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I120" s="2" t="inlineStr"/>
@@ -5652,7 +5652,7 @@
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Salmos 27:14. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I121" s="2" t="inlineStr"/>
@@ -5695,7 +5695,7 @@
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Isaías 12:2. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I122" s="2" t="inlineStr"/>
@@ -5738,7 +5738,7 @@
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com 2 Crônicas 20:15. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I123" s="2" t="inlineStr"/>
@@ -5781,7 +5781,7 @@
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Salmos 46:1-2. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I124" s="2" t="inlineStr"/>
@@ -5824,7 +5824,7 @@
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Marcos 4:39-40. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I125" s="2" t="inlineStr"/>
@@ -5867,7 +5867,7 @@
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Mateus 14:29-31. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I126" s="2" t="inlineStr"/>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Salmos 112:7. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I127" s="2" t="inlineStr"/>
@@ -5953,7 +5953,7 @@
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Lucas 1:37. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I128" s="2" t="inlineStr"/>
@@ -5996,7 +5996,7 @@
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Juízes 6:12. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I129" s="2" t="inlineStr"/>
@@ -6039,7 +6039,7 @@
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Salmos 31:24. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I130" s="2" t="inlineStr"/>
@@ -6082,7 +6082,7 @@
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Ester 4:14. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I131" s="2" t="inlineStr"/>
@@ -6125,7 +6125,7 @@
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Daniel 3:17-18. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I132" s="2" t="inlineStr"/>
@@ -6168,7 +6168,7 @@
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Atos 18:9-10. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I133" s="2" t="inlineStr"/>
@@ -6211,7 +6211,7 @@
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Salmos 138:3. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I134" s="2" t="inlineStr"/>
@@ -6254,7 +6254,7 @@
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Isaías 54:17. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I135" s="2" t="inlineStr"/>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Provérbios 3:25-26. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I136" s="2" t="inlineStr"/>
@@ -6340,7 +6340,7 @@
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com Neemias 4:14. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I137" s="2" t="inlineStr"/>
@@ -6383,7 +6383,7 @@
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: medo e coragem 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #medo</t>
+          <t>Oração da noite: medo e coragem 🌙 Para fechar o dia com 2 Coríntios 12:9-10. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #medo</t>
         </is>
       </c>
       <c r="I138" s="2" t="inlineStr"/>
@@ -6426,7 +6426,7 @@
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Lamentações 3:22-23. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I139" s="2" t="inlineStr"/>
@@ -6469,7 +6469,7 @@
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Jeremias 29:11. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I140" s="2" t="inlineStr"/>
@@ -6512,7 +6512,7 @@
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Romanos 15:13. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I141" s="2" t="inlineStr"/>
@@ -6555,7 +6555,7 @@
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Salmos 42:11. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I142" s="2" t="inlineStr"/>
@@ -6598,7 +6598,7 @@
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Isaías 43:19. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I143" s="2" t="inlineStr"/>
@@ -6641,7 +6641,7 @@
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Romanos 5:3-5. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I144" s="2" t="inlineStr"/>
@@ -6684,7 +6684,7 @@
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com 2 Coríntios 4:16-18. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I145" s="2" t="inlineStr"/>
@@ -6727,7 +6727,7 @@
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Salmos 30:5. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I146" s="2" t="inlineStr"/>
@@ -6770,7 +6770,7 @@
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Habacuque 3:17-18. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I147" s="2" t="inlineStr"/>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Hebreus 6:19. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I148" s="2" t="inlineStr"/>
@@ -6856,7 +6856,7 @@
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Salmos 40:1-2. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I149" s="2" t="inlineStr"/>
@@ -6899,7 +6899,7 @@
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Isaías 61:3. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I150" s="2" t="inlineStr"/>
@@ -6942,7 +6942,7 @@
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Romanos 8:18. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I151" s="2" t="inlineStr"/>
@@ -6985,7 +6985,7 @@
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Miqueias 7:8. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I152" s="2" t="inlineStr"/>
@@ -7028,7 +7028,7 @@
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Salmos 147:3. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I153" s="2" t="inlineStr"/>
@@ -7071,7 +7071,7 @@
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Joel 2:25. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I154" s="2" t="inlineStr"/>
@@ -7114,7 +7114,7 @@
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Jó 42:10. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I155" s="2" t="inlineStr"/>
@@ -7157,7 +7157,7 @@
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Salmos 34:18. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I156" s="2" t="inlineStr"/>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Apocalipse 21:4. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I157" s="2" t="inlineStr"/>
@@ -7243,7 +7243,7 @@
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Romanos 12:12. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I158" s="2" t="inlineStr"/>
@@ -7286,7 +7286,7 @@
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Isaías 40:29. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I159" s="2" t="inlineStr"/>
@@ -7329,7 +7329,7 @@
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Salmos 71:20. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I160" s="2" t="inlineStr"/>
@@ -7372,7 +7372,7 @@
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com 1 Pedro 1:3. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I161" s="2" t="inlineStr"/>
@@ -7415,7 +7415,7 @@
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Gênesis 50:20. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I162" s="2" t="inlineStr"/>
@@ -7458,7 +7458,7 @@
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Salmos 126:5-6. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I163" s="2" t="inlineStr"/>
@@ -7501,7 +7501,7 @@
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Isaías 9:2. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I164" s="2" t="inlineStr"/>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Salmos 62:5. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I165" s="2" t="inlineStr"/>
@@ -7587,7 +7587,7 @@
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Isaías 35:3-4. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I166" s="2" t="inlineStr"/>
@@ -7630,7 +7630,7 @@
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com 2 Coríntios 4:8-9. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I167" s="2" t="inlineStr"/>
@@ -7673,7 +7673,7 @@
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Salmos 33:20-22. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I168" s="2" t="inlineStr"/>
@@ -7716,7 +7716,7 @@
       </c>
       <c r="H169" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: esperança em tempos difíceis 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #esperanca</t>
+          <t>Oração da noite: esperança em tempos difíceis 🌙 Para fechar o dia com Mateus 28:20. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #esperanca</t>
         </is>
       </c>
       <c r="I169" s="2" t="inlineStr"/>
@@ -7759,7 +7759,7 @@
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Efésios 4:32. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I170" s="2" t="inlineStr"/>
@@ -7802,7 +7802,7 @@
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Colossenses 3:13. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I171" s="2" t="inlineStr"/>
@@ -7845,7 +7845,7 @@
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Mateus 6:14-15. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I172" s="2" t="inlineStr"/>
@@ -7888,7 +7888,7 @@
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Mateus 18:21-22. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I173" s="2" t="inlineStr"/>
@@ -7931,7 +7931,7 @@
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com 1 João 1:9. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I174" s="2" t="inlineStr"/>
@@ -7974,7 +7974,7 @@
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Salmos 103:12. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I175" s="2" t="inlineStr"/>
@@ -8017,7 +8017,7 @@
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Isaías 1:18. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I176" s="2" t="inlineStr"/>
@@ -8060,7 +8060,7 @@
       </c>
       <c r="H177" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Lucas 15:20. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I177" s="2" t="inlineStr"/>
@@ -8103,7 +8103,7 @@
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Lucas 23:34. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I178" s="2" t="inlineStr"/>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="H179" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Miqueias 7:18-19. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I179" s="2" t="inlineStr"/>
@@ -8189,7 +8189,7 @@
       </c>
       <c r="H180" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Romanos 12:17-19. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I180" s="2" t="inlineStr"/>
@@ -8232,7 +8232,7 @@
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Salmos 32:1-2. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I181" s="2" t="inlineStr"/>
@@ -8275,7 +8275,7 @@
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Marcos 11:25. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I182" s="2" t="inlineStr"/>
@@ -8318,7 +8318,7 @@
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Hebreus 8:12. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I183" s="2" t="inlineStr"/>
@@ -8361,7 +8361,7 @@
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Gênesis 45:4-5. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I184" s="2" t="inlineStr"/>
@@ -8404,7 +8404,7 @@
       </c>
       <c r="H185" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Provérbios 19:11. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I185" s="2" t="inlineStr"/>
@@ -8447,7 +8447,7 @@
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com 2 Coríntios 5:17. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I186" s="2" t="inlineStr"/>
@@ -8490,7 +8490,7 @@
       </c>
       <c r="H187" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Romanos 8:1. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I187" s="2" t="inlineStr"/>
@@ -8533,7 +8533,7 @@
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Lucas 6:37. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I188" s="2" t="inlineStr"/>
@@ -8576,7 +8576,7 @@
       </c>
       <c r="H189" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Salmos 51:10. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I189" s="2" t="inlineStr"/>
@@ -8619,7 +8619,7 @@
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Atos 3:19. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I190" s="2" t="inlineStr"/>
@@ -8662,7 +8662,7 @@
       </c>
       <c r="H191" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Mateus 5:23-24. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I191" s="2" t="inlineStr"/>
@@ -8705,7 +8705,7 @@
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Efésios 4:26-27. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I192" s="2" t="inlineStr"/>
@@ -8748,7 +8748,7 @@
       </c>
       <c r="H193" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Lucas 7:47. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I193" s="2" t="inlineStr"/>
@@ -8791,7 +8791,7 @@
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com João 8:10-11. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I194" s="2" t="inlineStr"/>
@@ -8834,7 +8834,7 @@
       </c>
       <c r="H195" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Isaías 43:25. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I195" s="2" t="inlineStr"/>
@@ -8877,7 +8877,7 @@
       </c>
       <c r="H196" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Salmos 130:3-4. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I196" s="2" t="inlineStr"/>
@@ -8920,7 +8920,7 @@
       </c>
       <c r="H197" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Colossenses 2:13-14. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I197" s="2" t="inlineStr"/>
@@ -8963,7 +8963,7 @@
       </c>
       <c r="H198" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com 1 Pedro 3:9. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I198" s="2" t="inlineStr"/>
@@ -9006,7 +9006,7 @@
       </c>
       <c r="H199" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: perdão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #perdao</t>
+          <t>Oração da noite: perdão 🌙 Para fechar o dia com Lucas 17:3-4. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #perdao</t>
         </is>
       </c>
       <c r="I199" s="2" t="inlineStr"/>
@@ -9049,7 +9049,7 @@
       </c>
       <c r="H200" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Josué 24:15. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I200" s="2" t="inlineStr"/>
@@ -9092,7 +9092,7 @@
       </c>
       <c r="H201" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Salmos 127:1. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I201" s="2" t="inlineStr"/>
@@ -9135,7 +9135,7 @@
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Provérbios 22:6. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I202" s="2" t="inlineStr"/>
@@ -9178,7 +9178,7 @@
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Efésios 6:1-3. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I203" s="2" t="inlineStr"/>
@@ -9221,7 +9221,7 @@
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Eclesiastes 4:9-10. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I204" s="2" t="inlineStr"/>
@@ -9264,7 +9264,7 @@
       </c>
       <c r="H205" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Eclesiastes 4:12. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I205" s="2" t="inlineStr"/>
@@ -9307,7 +9307,7 @@
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Rute 1:16-17. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I206" s="2" t="inlineStr"/>
@@ -9350,7 +9350,7 @@
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Provérbios 17:17. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I207" s="2" t="inlineStr"/>
@@ -9393,7 +9393,7 @@
       </c>
       <c r="H208" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Colossenses 3:14. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I208" s="2" t="inlineStr"/>
@@ -9436,7 +9436,7 @@
       </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com 1 Coríntios 13:4-5. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I209" s="2" t="inlineStr"/>
@@ -9479,7 +9479,7 @@
       </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Gênesis 2:24. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I210" s="2" t="inlineStr"/>
@@ -9522,7 +9522,7 @@
       </c>
       <c r="H211" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Provérbios 31:10-11. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I211" s="2" t="inlineStr"/>
@@ -9565,7 +9565,7 @@
       </c>
       <c r="H212" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Efésios 5:25. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I212" s="2" t="inlineStr"/>
@@ -9608,7 +9608,7 @@
       </c>
       <c r="H213" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Salmos 133:1. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I213" s="2" t="inlineStr"/>
@@ -9651,7 +9651,7 @@
       </c>
       <c r="H214" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Provérbios 15:1. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I214" s="2" t="inlineStr"/>
@@ -9694,7 +9694,7 @@
       </c>
       <c r="H215" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Tiago 1:19. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I215" s="2" t="inlineStr"/>
@@ -9737,7 +9737,7 @@
       </c>
       <c r="H216" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com 1 Pedro 4:8. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I216" s="2" t="inlineStr"/>
@@ -9780,7 +9780,7 @@
       </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Malaquias 4:6. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I217" s="2" t="inlineStr"/>
@@ -9823,7 +9823,7 @@
       </c>
       <c r="H218" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Salmos 68:6. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I218" s="2" t="inlineStr"/>
@@ -9866,7 +9866,7 @@
       </c>
       <c r="H219" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Provérbios 27:17. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I219" s="2" t="inlineStr"/>
@@ -9909,7 +9909,7 @@
       </c>
       <c r="H220" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Romanos 12:10. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I220" s="2" t="inlineStr"/>
@@ -9952,7 +9952,7 @@
       </c>
       <c r="H221" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com 1 Tessalonicenses 5:11. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I221" s="2" t="inlineStr"/>
@@ -9995,7 +9995,7 @@
       </c>
       <c r="H222" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Lucas 2:51-52. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I222" s="2" t="inlineStr"/>
@@ -10038,7 +10038,7 @@
       </c>
       <c r="H223" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Provérbios 18:24. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I223" s="2" t="inlineStr"/>
@@ -10081,7 +10081,7 @@
       </c>
       <c r="H224" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com João 15:13. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I224" s="2" t="inlineStr"/>
@@ -10124,7 +10124,7 @@
       </c>
       <c r="H225" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Gálatas 6:2. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I225" s="2" t="inlineStr"/>
@@ -10167,7 +10167,7 @@
       </c>
       <c r="H226" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Filipenses 2:3-4. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I226" s="2" t="inlineStr"/>
@@ -10210,7 +10210,7 @@
       </c>
       <c r="H227" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Salmos 103:13. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I227" s="2" t="inlineStr"/>
@@ -10253,7 +10253,7 @@
       </c>
       <c r="H228" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Isaías 49:15. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I228" s="2" t="inlineStr"/>
@@ -10296,7 +10296,7 @@
       </c>
       <c r="H229" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com 1 João 4:11. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I229" s="2" t="inlineStr"/>
@@ -10339,7 +10339,7 @@
       </c>
       <c r="H230" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: família e relacionamentos 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #familia</t>
+          <t>Oração da noite: família e relacionamentos 🌙 Para fechar o dia com Hebreus 13:1. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #familia</t>
         </is>
       </c>
       <c r="I230" s="2" t="inlineStr"/>
@@ -10382,7 +10382,7 @@
       </c>
       <c r="H231" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com 1 Tessalonicenses 5:18. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I231" s="2" t="inlineStr"/>
@@ -10425,7 +10425,7 @@
       </c>
       <c r="H232" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Salmos 118:24. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I232" s="2" t="inlineStr"/>
@@ -10468,7 +10468,7 @@
       </c>
       <c r="H233" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Salmos 100:4. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I233" s="2" t="inlineStr"/>
@@ -10511,7 +10511,7 @@
       </c>
       <c r="H234" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Colossenses 3:15. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I234" s="2" t="inlineStr"/>
@@ -10554,7 +10554,7 @@
       </c>
       <c r="H235" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Salmos 103:2. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I235" s="2" t="inlineStr"/>
@@ -10597,7 +10597,7 @@
       </c>
       <c r="H236" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Lucas 17:15-16. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I236" s="2" t="inlineStr"/>
@@ -10640,7 +10640,7 @@
       </c>
       <c r="H237" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Tiago 1:17. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I237" s="2" t="inlineStr"/>
@@ -10683,7 +10683,7 @@
       </c>
       <c r="H238" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Salmos 136:1. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I238" s="2" t="inlineStr"/>
@@ -10726,7 +10726,7 @@
       </c>
       <c r="H239" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Filipenses 4:11-12. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I239" s="2" t="inlineStr"/>
@@ -10769,7 +10769,7 @@
       </c>
       <c r="H240" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Salmos 9:1. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I240" s="2" t="inlineStr"/>
@@ -10812,7 +10812,7 @@
       </c>
       <c r="H241" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Salmos 107:1. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I241" s="2" t="inlineStr"/>
@@ -10855,7 +10855,7 @@
       </c>
       <c r="H242" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Efésios 5:20. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I242" s="2" t="inlineStr"/>
@@ -10898,7 +10898,7 @@
       </c>
       <c r="H243" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Hebreus 12:28. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I243" s="2" t="inlineStr"/>
@@ -10941,7 +10941,7 @@
       </c>
       <c r="H244" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Salmos 92:1-2. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I244" s="2" t="inlineStr"/>
@@ -10984,7 +10984,7 @@
       </c>
       <c r="H245" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com 1 Crônicas 16:34. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I245" s="2" t="inlineStr"/>
@@ -11027,7 +11027,7 @@
       </c>
       <c r="H246" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com 2 Coríntios 9:15. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I246" s="2" t="inlineStr"/>
@@ -11070,7 +11070,7 @@
       </c>
       <c r="H247" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Salmos 34:1. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I247" s="2" t="inlineStr"/>
@@ -11113,7 +11113,7 @@
       </c>
       <c r="H248" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Daniel 6:10. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I248" s="2" t="inlineStr"/>
@@ -11156,7 +11156,7 @@
       </c>
       <c r="H249" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Salmos 50:23. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I249" s="2" t="inlineStr"/>
@@ -11199,7 +11199,7 @@
       </c>
       <c r="H250" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Romanos 1:21. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I250" s="2" t="inlineStr"/>
@@ -11242,7 +11242,7 @@
       </c>
       <c r="H251" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Salmos 16:6. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I251" s="2" t="inlineStr"/>
@@ -11285,7 +11285,7 @@
       </c>
       <c r="H252" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Salmos 145:9. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I252" s="2" t="inlineStr"/>
@@ -11328,7 +11328,7 @@
       </c>
       <c r="H253" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com João 6:11. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I253" s="2" t="inlineStr"/>
@@ -11371,7 +11371,7 @@
       </c>
       <c r="H254" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Salmos 95:2. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I254" s="2" t="inlineStr"/>
@@ -11414,7 +11414,7 @@
       </c>
       <c r="H255" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Lamentações 3:24. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I255" s="2" t="inlineStr"/>
@@ -11457,7 +11457,7 @@
       </c>
       <c r="H256" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Salmos 116:12. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I256" s="2" t="inlineStr"/>
@@ -11500,7 +11500,7 @@
       </c>
       <c r="H257" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Atos 16:25. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I257" s="2" t="inlineStr"/>
@@ -11543,7 +11543,7 @@
       </c>
       <c r="H258" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Salmos 103:3-5. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I258" s="2" t="inlineStr"/>
@@ -11586,7 +11586,7 @@
       </c>
       <c r="H259" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Salmos 65:11. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I259" s="2" t="inlineStr"/>
@@ -11629,7 +11629,7 @@
       </c>
       <c r="H260" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: gratidão 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #gratidao</t>
+          <t>Oração da noite: gratidão 🌙 Para fechar o dia com Neemias 8:10. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #gratidao</t>
         </is>
       </c>
       <c r="I260" s="2" t="inlineStr"/>
@@ -11672,7 +11672,7 @@
       </c>
       <c r="H261" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Colossenses 3:23. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I261" s="2" t="inlineStr"/>
@@ -11715,7 +11715,7 @@
       </c>
       <c r="H262" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Provérbios 16:3. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I262" s="2" t="inlineStr"/>
@@ -11758,7 +11758,7 @@
       </c>
       <c r="H263" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Efésios 2:10. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I263" s="2" t="inlineStr"/>
@@ -11801,7 +11801,7 @@
       </c>
       <c r="H264" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Jeremias 1:5. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I264" s="2" t="inlineStr"/>
@@ -11844,7 +11844,7 @@
       </c>
       <c r="H265" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Provérbios 14:23. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I265" s="2" t="inlineStr"/>
@@ -11887,7 +11887,7 @@
       </c>
       <c r="H266" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Eclesiastes 9:10. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I266" s="2" t="inlineStr"/>
@@ -11930,7 +11930,7 @@
       </c>
       <c r="H267" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Provérbios 22:29. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I267" s="2" t="inlineStr"/>
@@ -11973,7 +11973,7 @@
       </c>
       <c r="H268" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Filipenses 1:6. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I268" s="2" t="inlineStr"/>
@@ -12016,7 +12016,7 @@
       </c>
       <c r="H269" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Gálatas 6:9. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I269" s="2" t="inlineStr"/>
@@ -12059,7 +12059,7 @@
       </c>
       <c r="H270" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Salmos 90:17. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I270" s="2" t="inlineStr"/>
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H271" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Romanos 12:6-8. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I271" s="2" t="inlineStr"/>
@@ -12145,7 +12145,7 @@
       </c>
       <c r="H272" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com 1 Pedro 4:10. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I272" s="2" t="inlineStr"/>
@@ -12188,7 +12188,7 @@
       </c>
       <c r="H273" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Provérbios 6:6-8. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I273" s="2" t="inlineStr"/>
@@ -12231,7 +12231,7 @@
       </c>
       <c r="H274" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Mateus 25:21. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I274" s="2" t="inlineStr"/>
@@ -12274,7 +12274,7 @@
       </c>
       <c r="H275" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Neemias 2:20. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I275" s="2" t="inlineStr"/>
@@ -12317,7 +12317,7 @@
       </c>
       <c r="H276" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Provérbios 13:4. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I276" s="2" t="inlineStr"/>
@@ -12360,7 +12360,7 @@
       </c>
       <c r="H277" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Mateus 5:14-16. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I277" s="2" t="inlineStr"/>
@@ -12403,7 +12403,7 @@
       </c>
       <c r="H278" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com 1 Coríntios 15:58. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I278" s="2" t="inlineStr"/>
@@ -12446,7 +12446,7 @@
       </c>
       <c r="H279" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Deuteronômio 8:18. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I279" s="2" t="inlineStr"/>
@@ -12489,7 +12489,7 @@
       </c>
       <c r="H280" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Provérbios 10:4. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I280" s="2" t="inlineStr"/>
@@ -12532,7 +12532,7 @@
       </c>
       <c r="H281" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Eclesiastes 3:1. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I281" s="2" t="inlineStr"/>
@@ -12575,7 +12575,7 @@
       </c>
       <c r="H282" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com 2 Tessalonicenses 3:10-13. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I282" s="2" t="inlineStr"/>
@@ -12618,7 +12618,7 @@
       </c>
       <c r="H283" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Isaías 64:8. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I283" s="2" t="inlineStr"/>
@@ -12661,7 +12661,7 @@
       </c>
       <c r="H284" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Atos 20:35. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I284" s="2" t="inlineStr"/>
@@ -12704,7 +12704,7 @@
       </c>
       <c r="H285" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Provérbios 16:9. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I285" s="2" t="inlineStr"/>
@@ -12747,7 +12747,7 @@
       </c>
       <c r="H286" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Habacuque 2:2-3. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I286" s="2" t="inlineStr"/>
@@ -12790,7 +12790,7 @@
       </c>
       <c r="H287" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Gênesis 39:2-3. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I287" s="2" t="inlineStr"/>
@@ -12833,7 +12833,7 @@
       </c>
       <c r="H288" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com 1 Coríntios 10:31. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I288" s="2" t="inlineStr"/>
@@ -12876,7 +12876,7 @@
       </c>
       <c r="H289" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Salmos 37:5. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I289" s="2" t="inlineStr"/>
@@ -12919,7 +12919,7 @@
       </c>
       <c r="H290" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Zacarias 4:10. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I290" s="2" t="inlineStr"/>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="H291" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: propósito e trabalho 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #proposito</t>
+          <t>Oração da noite: propósito e trabalho 🌙 Para fechar o dia com Mateus 6:33. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #proposito</t>
         </is>
       </c>
       <c r="I291" s="2" t="inlineStr"/>
@@ -13005,7 +13005,7 @@
       </c>
       <c r="H292" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Tiago 1:5. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I292" s="2" t="inlineStr"/>
@@ -13048,7 +13048,7 @@
       </c>
       <c r="H293" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Provérbios 3:5-6. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I293" s="2" t="inlineStr"/>
@@ -13091,7 +13091,7 @@
       </c>
       <c r="H294" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Salmos 119:105. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I294" s="2" t="inlineStr"/>
@@ -13134,7 +13134,7 @@
       </c>
       <c r="H295" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Provérbios 1:7. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I295" s="2" t="inlineStr"/>
@@ -13177,7 +13177,7 @@
       </c>
       <c r="H296" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Provérbios 11:14. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I296" s="2" t="inlineStr"/>
@@ -13220,7 +13220,7 @@
       </c>
       <c r="H297" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Salmos 32:8. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I297" s="2" t="inlineStr"/>
@@ -13263,7 +13263,7 @@
       </c>
       <c r="H298" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Provérbios 4:23. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I298" s="2" t="inlineStr"/>
@@ -13306,7 +13306,7 @@
       </c>
       <c r="H299" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Isaías 30:21. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I299" s="2" t="inlineStr"/>
@@ -13349,7 +13349,7 @@
       </c>
       <c r="H300" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Provérbios 2:6. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I300" s="2" t="inlineStr"/>
@@ -13392,7 +13392,7 @@
       </c>
       <c r="H301" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Tiago 3:17. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I301" s="2" t="inlineStr"/>
@@ -13435,7 +13435,7 @@
       </c>
       <c r="H302" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Provérbios 15:22. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I302" s="2" t="inlineStr"/>
@@ -13478,7 +13478,7 @@
       </c>
       <c r="H303" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Salmos 25:4-5. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I303" s="2" t="inlineStr"/>
@@ -13521,7 +13521,7 @@
       </c>
       <c r="H304" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Provérbios 16:16. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I304" s="2" t="inlineStr"/>
@@ -13564,7 +13564,7 @@
       </c>
       <c r="H305" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Colossenses 3:16. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I305" s="2" t="inlineStr"/>
@@ -13607,7 +13607,7 @@
       </c>
       <c r="H306" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Provérbios 14:12. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I306" s="2" t="inlineStr"/>
@@ -13650,7 +13650,7 @@
       </c>
       <c r="H307" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com 1 Reis 3:9. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I307" s="2" t="inlineStr"/>
@@ -13693,7 +13693,7 @@
       </c>
       <c r="H308" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Provérbios 19:21. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I308" s="2" t="inlineStr"/>
@@ -13736,7 +13736,7 @@
       </c>
       <c r="H309" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Romanos 12:2. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I309" s="2" t="inlineStr"/>
@@ -13779,7 +13779,7 @@
       </c>
       <c r="H310" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Salmos 1:1-3. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I310" s="2" t="inlineStr"/>
@@ -13822,7 +13822,7 @@
       </c>
       <c r="H311" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Provérbios 13:20. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I311" s="2" t="inlineStr"/>
@@ -13865,7 +13865,7 @@
       </c>
       <c r="H312" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Eclesiastes 7:8. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I312" s="2" t="inlineStr"/>
@@ -13908,7 +13908,7 @@
       </c>
       <c r="H313" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Provérbios 12:15. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I313" s="2" t="inlineStr"/>
@@ -13951,7 +13951,7 @@
       </c>
       <c r="H314" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Salmos 37:23. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I314" s="2" t="inlineStr"/>
@@ -13994,7 +13994,7 @@
       </c>
       <c r="H315" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Provérbios 21:5. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I315" s="2" t="inlineStr"/>
@@ -14037,7 +14037,7 @@
       </c>
       <c r="H316" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Filipenses 1:9-10. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I316" s="2" t="inlineStr"/>
@@ -14080,7 +14080,7 @@
       </c>
       <c r="H317" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Provérbios 18:13. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I317" s="2" t="inlineStr"/>
@@ -14123,7 +14123,7 @@
       </c>
       <c r="H318" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Mateus 7:24-25. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I318" s="2" t="inlineStr"/>
@@ -14166,7 +14166,7 @@
       </c>
       <c r="H319" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Salmos 111:10. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I319" s="2" t="inlineStr"/>
@@ -14209,7 +14209,7 @@
       </c>
       <c r="H320" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Provérbios 27:12. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I320" s="2" t="inlineStr"/>
@@ -14252,7 +14252,7 @@
       </c>
       <c r="H321" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Eclesiastes 12:13. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I321" s="2" t="inlineStr"/>
@@ -14295,7 +14295,7 @@
       </c>
       <c r="H322" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: sabedoria e decisões 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #sabedoria</t>
+          <t>Oração da noite: sabedoria e decisões 🌙 Para fechar o dia com Daniel 2:20-21. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #sabedoria</t>
         </is>
       </c>
       <c r="I322" s="2" t="inlineStr"/>
@@ -14338,7 +14338,7 @@
       </c>
       <c r="H323" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Filipenses 4:13. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I323" s="2" t="inlineStr"/>
@@ -14381,7 +14381,7 @@
       </c>
       <c r="H324" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Hebreus 12:1-2. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I324" s="2" t="inlineStr"/>
@@ -14424,7 +14424,7 @@
       </c>
       <c r="H325" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Salmos 27:13. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I325" s="2" t="inlineStr"/>
@@ -14467,7 +14467,7 @@
       </c>
       <c r="H326" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Tiago 1:2-4. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I326" s="2" t="inlineStr"/>
@@ -14510,7 +14510,7 @@
       </c>
       <c r="H327" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Provérbios 24:16. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I327" s="2" t="inlineStr"/>
@@ -14553,7 +14553,7 @@
       </c>
       <c r="H328" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com 2 Timóteo 4:7. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I328" s="2" t="inlineStr"/>
@@ -14596,7 +14596,7 @@
       </c>
       <c r="H329" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Salmos 18:32. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I329" s="2" t="inlineStr"/>
@@ -14639,7 +14639,7 @@
       </c>
       <c r="H330" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Salmos 66:10-12. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I330" s="2" t="inlineStr"/>
@@ -14682,7 +14682,7 @@
       </c>
       <c r="H331" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Salmos 73:26. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I331" s="2" t="inlineStr"/>
@@ -14725,7 +14725,7 @@
       </c>
       <c r="H332" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Isaías 41:13. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I332" s="2" t="inlineStr"/>
@@ -14768,7 +14768,7 @@
       </c>
       <c r="H333" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com 1 Coríntios 16:13. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I333" s="2" t="inlineStr"/>
@@ -14811,7 +14811,7 @@
       </c>
       <c r="H334" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Efésios 6:10. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I334" s="2" t="inlineStr"/>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="H335" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Salmos 28:7. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I335" s="2" t="inlineStr"/>
@@ -14897,7 +14897,7 @@
       </c>
       <c r="H336" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Hebreus 10:36. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I336" s="2" t="inlineStr"/>
@@ -14940,7 +14940,7 @@
       </c>
       <c r="H337" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Zacarias 4:6. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I337" s="2" t="inlineStr"/>
@@ -14983,7 +14983,7 @@
       </c>
       <c r="H338" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Isaías 50:7. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I338" s="2" t="inlineStr"/>
@@ -15026,7 +15026,7 @@
       </c>
       <c r="H339" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Salmos 138:7. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I339" s="2" t="inlineStr"/>
@@ -15069,7 +15069,7 @@
       </c>
       <c r="H340" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Neemias 6:3. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I340" s="2" t="inlineStr"/>
@@ -15112,7 +15112,7 @@
       </c>
       <c r="H341" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Tiago 1:12. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I341" s="2" t="inlineStr"/>
@@ -15155,7 +15155,7 @@
       </c>
       <c r="H342" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Salmos 46:5. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I342" s="2" t="inlineStr"/>
@@ -15198,7 +15198,7 @@
       </c>
       <c r="H343" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Hebreus 12:11. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I343" s="2" t="inlineStr"/>
@@ -15241,7 +15241,7 @@
       </c>
       <c r="H344" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Lucas 18:1. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I344" s="2" t="inlineStr"/>
@@ -15284,7 +15284,7 @@
       </c>
       <c r="H345" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Salmos 37:24. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I345" s="2" t="inlineStr"/>
@@ -15327,7 +15327,7 @@
       </c>
       <c r="H346" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com 2 Coríntios 4:7. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I346" s="2" t="inlineStr"/>
@@ -15370,7 +15370,7 @@
       </c>
       <c r="H347" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Josué 14:11. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I347" s="2" t="inlineStr"/>
@@ -15413,7 +15413,7 @@
       </c>
       <c r="H348" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Isaías 40:28. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I348" s="2" t="inlineStr"/>
@@ -15456,7 +15456,7 @@
       </c>
       <c r="H349" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Romanos 8:37. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I349" s="2" t="inlineStr"/>
@@ -15499,7 +15499,7 @@
       </c>
       <c r="H350" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Habacuque 3:19. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I350" s="2" t="inlineStr"/>
@@ -15542,7 +15542,7 @@
       </c>
       <c r="H351" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com Apocalipse 2:10. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I351" s="2" t="inlineStr"/>
@@ -15585,7 +15585,7 @@
       </c>
       <c r="H352" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: força e perseverança 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
+          <t>Oração da noite: força e perseverança 🌙 Para fechar o dia com 2 Crônicas 15:7. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #forca</t>
         </is>
       </c>
       <c r="I352" s="2" t="inlineStr"/>
@@ -15628,7 +15628,7 @@
       </c>
       <c r="H353" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com João 3:16. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I353" s="2" t="inlineStr"/>
@@ -15671,7 +15671,7 @@
       </c>
       <c r="H354" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com 1 João 4:8. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I354" s="2" t="inlineStr"/>
@@ -15714,7 +15714,7 @@
       </c>
       <c r="H355" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Romanos 5:8. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I355" s="2" t="inlineStr"/>
@@ -15757,7 +15757,7 @@
       </c>
       <c r="H356" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Romanos 8:38-39. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I356" s="2" t="inlineStr"/>
@@ -15800,7 +15800,7 @@
       </c>
       <c r="H357" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com 1 João 4:19. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I357" s="2" t="inlineStr"/>
@@ -15843,7 +15843,7 @@
       </c>
       <c r="H358" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Jeremias 31:3. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I358" s="2" t="inlineStr"/>
@@ -15886,7 +15886,7 @@
       </c>
       <c r="H359" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com 1 Coríntios 13:7. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I359" s="2" t="inlineStr"/>
@@ -15929,7 +15929,7 @@
       </c>
       <c r="H360" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com 1 Coríntios 13:13. Escreva amém se essa oração é sua também. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I360" s="2" t="inlineStr"/>
@@ -15972,7 +15972,7 @@
       </c>
       <c r="H361" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Mateus 22:37-39. Comente o nome de quem você quer colocar nesta oração. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I361" s="2" t="inlineStr"/>
@@ -16015,7 +16015,7 @@
       </c>
       <c r="H362" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com João 13:34-35. Conte nos comentários pelo que você quer agradecer hoje. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I362" s="2" t="inlineStr"/>
@@ -16058,7 +16058,7 @@
       </c>
       <c r="H363" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Lucas 6:27-28. Deixe nos comentários o que você quer entregar a Deus esta noite. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I363" s="2" t="inlineStr"/>
@@ -16101,7 +16101,7 @@
       </c>
       <c r="H364" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Efésios 3:17-19. Marque alguém que precisa ouvir esta oração. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I364" s="2" t="inlineStr"/>
@@ -16144,7 +16144,7 @@
       </c>
       <c r="H365" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com 1 João 3:18. Comente seu pedido. Vamos orar juntos. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I365" s="2" t="inlineStr"/>
@@ -16187,7 +16187,7 @@
       </c>
       <c r="H366" s="2" t="inlineStr">
         <is>
-          <t>Oração da noite: amor 🌙 Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
+          <t>Oração da noite: amor 🌙 Para fechar o dia com Romanos 13:10. Deixe seu pedido de oração nos comentários. #oracaodanoite #oracao #fe #amor</t>
         </is>
       </c>
       <c r="I366" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Nova contagem, gancho e CTA nos vídeos de 21/10 a 19/12
A pílula e a linha "Amanhã tem o dia" passam a contar a partir de 15/10 (Dia 1).
Cada vídeo ganha um gancho de 1,3 s no início e uma tela final com motivo
concreto para seguir. A legenda da manhã acompanha a nova contagem nesses dias.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Eevu1kG1RwxjevYg68LqvH
</commit_message>
<xml_diff>
--- a/legendas-365.xlsx
+++ b/legendas-365.xlsx
@@ -773,7 +773,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Dia 294 de 365. João 15:9: Permanecei no meu amor. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 7 de 365. João 15:9: Permanecei no meu amor. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Dia 295 de 365. Efésios 2:4-5: Rico em misericórdia. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 8 de 365. Efésios 2:4-5: Rico em misericórdia. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Dia 296 de 365. Romanos 12:9: O amor seja sem fingimento. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 9 de 365. Romanos 12:9: O amor seja sem fingimento. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Dia 297 de 365. Provérbios 10:12: O ódio provoca brigas. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 10 de 365. Provérbios 10:12: O ódio provoca brigas. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -945,7 +945,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Dia 298 de 365. 1 João 4:20: Quem diz que ama a Deus. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 11 de 365. 1 João 4:20: Quem diz que ama a Deus. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Dia 299 de 365. Salmos 86:15: Lento para a ira, grande em amor. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 12 de 365. Salmos 86:15: Lento para a ira, grande em amor. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Dia 300 de 365. Oseias 11:4: Atraí-os com cordas de amor. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 13 de 365. Oseias 11:4: Atraí-os com cordas de amor. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Dia 301 de 365. Marcos 10:21: Jesus olhou para ele e o amou. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 14 de 365. Marcos 10:21: Jesus olhou para ele e o amou. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Dia 302 de 365. João 21:17: Tu sabes que eu te amo. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 15 de 365. João 21:17: Tu sabes que eu te amo. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Dia 303 de 365. Tito 3:4-5: A bondade e o amor de Deus apareceram. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 16 de 365. Tito 3:4-5: A bondade e o amor de Deus apareceram. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Dia 304 de 365. 1 Coríntios 16:14: Todas as vossas coisas sejam feitas com amor. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 17 de 365. 1 Coríntios 16:14: Todas as vossas coisas sejam feitas com amor. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Dia 305 de 365. Jeremias 33:3: Clama a mim, e responder-te-ei. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 18 de 365. Jeremias 33:3: Clama a mim, e responder-te-ei. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Dia 306 de 365. Mateus 7:7-8: Pedi, buscai, batei. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 19 de 365. Mateus 7:7-8: Pedi, buscai, batei. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Dia 307 de 365. 1 Tessalonicenses 5:17: Orai sem cessar. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 20 de 365. 1 Tessalonicenses 5:17: Orai sem cessar. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Dia 308 de 365. Filipenses 4:19: O meu Deus suprirá. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 21 de 365. Filipenses 4:19: O meu Deus suprirá. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Dia 309 de 365. Salmos 37:4: Deleita-te no Senhor. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 22 de 365. Salmos 37:4: Deleita-te no Senhor. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Dia 310 de 365. Salmos 56:8: Deus guarda as suas lágrimas. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 23 de 365. Salmos 56:8: Deus guarda as suas lágrimas. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Dia 311 de 365. Marcos 11:24: Crede que recebestes. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 24 de 365. Marcos 11:24: Crede que recebestes. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Dia 312 de 365. Salmos 145:18: Perto está o Senhor. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 25 de 365. Salmos 145:18: Perto está o Senhor. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Dia 313 de 365. Mateus 6:6: Entre no seu quarto e feche a porta. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 26 de 365. Mateus 6:6: Entre no seu quarto e feche a porta. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Dia 314 de 365. Romanos 8:26: Quando você não sabe o que orar. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 27 de 365. Romanos 8:26: Quando você não sabe o que orar. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Dia 315 de 365. Hebreus 4:16: Cheguemos com confiança ao trono da graça. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 28 de 365. Hebreus 4:16: Cheguemos com confiança ao trono da graça. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Dia 316 de 365. Salmos 62:8: Derramai perante Ele o vosso coração. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 29 de 365. Salmos 62:8: Derramai perante Ele o vosso coração. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Dia 317 de 365. Tiago 5:16: A oração do justo pode muito. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 30 de 365. Tiago 5:16: A oração do justo pode muito. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Dia 318 de 365. Mateus 6:9-10: A oração que Jesus ensinou. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 31 de 365. Mateus 6:9-10: A oração que Jesus ensinou. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1848,7 +1848,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Dia 319 de 365. Salmos 5:3: De manhã ouvirás a minha voz. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 32 de 365. Salmos 5:3: De manhã ouvirás a minha voz. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Dia 320 de 365. Lucas 22:42: Não a minha vontade, mas a tua. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 33 de 365. Lucas 22:42: Não a minha vontade, mas a tua. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Dia 321 de 365. 1 João 5:14: Se pedirmos segundo a sua vontade. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 34 de 365. 1 João 5:14: Se pedirmos segundo a sua vontade. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Dia 322 de 365. Salmos 20:7: Uns confiam em carros, outros em cavalos. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 35 de 365. Salmos 20:7: Uns confiam em carros, outros em cavalos. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Dia 323 de 365. Isaías 65:24: Antes que clamem, eu responderei. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 36 de 365. Isaías 65:24: Antes que clamem, eu responderei. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Dia 324 de 365. Neemias 1:4: Neemias chorou, jejuou e orou. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 37 de 365. Neemias 1:4: Neemias chorou, jejuou e orou. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Dia 325 de 365. Daniel 9:18: Não por nossas justiças. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 38 de 365. Daniel 9:18: Não por nossas justiças. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Dia 326 de 365. Salmos 37:7: Descansa no Senhor e espera nEle. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 39 de 365. Salmos 37:7: Descansa no Senhor e espera nEle. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Dia 327 de 365. Mateus 21:22: Tudo o que pedirdes em oração, crendo. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 40 de 365. Mateus 21:22: Tudo o que pedirdes em oração, crendo. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Dia 328 de 365. Salmos 141:2: Minha oração como incenso. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 41 de 365. Salmos 141:2: Minha oração como incenso. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2278,7 +2278,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Dia 329 de 365. Isaías 30:15: Na tranquilidade e na confiança. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 42 de 365. Isaías 30:15: Na tranquilidade e na confiança. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Dia 330 de 365. Salmos 9:10: Os que conhecem o teu nome confiarão em ti. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 43 de 365. Salmos 9:10: Os que conhecem o teu nome confiarão em ti. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Dia 331 de 365. Atos 12:5: A igreja orava por Pedro. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 44 de 365. Atos 12:5: A igreja orava por Pedro. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2407,7 +2407,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Dia 332 de 365. Lucas 11:9-10: Batei, e abrir-se-vos-á. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 45 de 365. Lucas 11:9-10: Batei, e abrir-se-vos-á. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2450,7 +2450,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Dia 333 de 365. Provérbios 29:25: O medo dos homens é um laço. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 46 de 365. Provérbios 29:25: O medo dos homens é um laço. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Dia 334 de 365. Salmos 57:1-2: À sombra das tuas asas. #fe #oracao #confianca #palavradodia</t>
+          <t>Dia 47 de 365. Salmos 57:1-2: À sombra das tuas asas. #fe #oracao #confianca #palavradodia</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Dia 335 de 365. Isaías 43:18: Não vos lembreis das coisas passadas. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 48 de 365. Isaías 43:18: Não vos lembreis das coisas passadas. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Dia 336 de 365. Filipenses 3:13-14: Esquecendo o que fica para trás. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 49 de 365. Filipenses 3:13-14: Esquecendo o que fica para trás. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Dia 337 de 365. Ezequiel 36:26: Um coração novo. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 50 de 365. Ezequiel 36:26: Um coração novo. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Dia 338 de 365. Apocalipse 21:5: Eis que faço novas todas as coisas. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 51 de 365. Apocalipse 21:5: Eis que faço novas todas as coisas. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Dia 339 de 365. Salmos 40:3: Um cântico novo. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 52 de 365. Salmos 40:3: Um cântico novo. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Dia 340 de 365. 2 Coríntios 1:20: Todas as promessas têm o sim nEle. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 53 de 365. 2 Coríntios 1:20: Todas as promessas têm o sim nEle. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Dia 341 de 365. Números 23:19: Deus não é homem para que minta. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 54 de 365. Números 23:19: Deus não é homem para que minta. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -2837,7 +2837,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Dia 342 de 365. Josué 21:45: Nenhuma palavra falhou. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 55 de 365. Josué 21:45: Nenhuma palavra falhou. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Dia 343 de 365. Lamentações 3:25: Bom é o Senhor para os que esperam por Ele. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 56 de 365. Lamentações 3:25: Bom é o Senhor para os que esperam por Ele. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -2923,7 +2923,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Dia 344 de 365. Isaías 55:10-11: A palavra de Deus não volta vazia. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 57 de 365. Isaías 55:10-11: A palavra de Deus não volta vazia. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Dia 345 de 365. Salmos 37:25: Nunca vi o justo desamparado. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 58 de 365. Salmos 37:25: Nunca vi o justo desamparado. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -3009,7 +3009,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Dia 346 de 365. Deuteronômio 7:9: O Deus fiel. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 59 de 365. Deuteronômio 7:9: O Deus fiel. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -3052,7 +3052,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Dia 347 de 365. Hebreus 10:23: Retenhamos firme a confissão da esperança. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 60 de 365. Hebreus 10:23: Retenhamos firme a confissão da esperança. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Dia 348 de 365. Jonas 2:10: Do fundo do peixe para a terra seca. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 61 de 365. Jonas 2:10: Do fundo do peixe para a terra seca. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Dia 349 de 365. Jonas 3:1: A palavra veio pela segunda vez. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 62 de 365. Jonas 3:1: A palavra veio pela segunda vez. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -3181,7 +3181,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Dia 350 de 365. Isaías 58:11: Como jardim regado. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 63 de 365. Isaías 58:11: Como jardim regado. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -3224,7 +3224,7 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Dia 351 de 365. Salmos 23:6: Bondade e misericórdia me seguirão. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 64 de 365. Salmos 23:6: Bondade e misericórdia me seguirão. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Dia 352 de 365. Gênesis 28:15: Eis que estou contigo. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 65 de 365. Gênesis 28:15: Eis que estou contigo. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -3310,7 +3310,7 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Dia 353 de 365. Isaías 42:3: A cana quebrada Ele não esmagará. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 66 de 365. Isaías 42:3: A cana quebrada Ele não esmagará. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Nova contagem, gancho e CTA até 15/01
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Eevu1kG1RwxjevYg68LqvH
</commit_message>
<xml_diff>
--- a/legendas-365.xlsx
+++ b/legendas-365.xlsx
@@ -3353,7 +3353,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Dia 354 de 365. Salmos 145:14: O Senhor sustenta os que caem. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 67 de 365. Salmos 145:14: O Senhor sustenta os que caem. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -3396,7 +3396,7 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Dia 355 de 365. Isaías 60:1: Levanta-te, resplandece. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 68 de 365. Isaías 60:1: Levanta-te, resplandece. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -3439,7 +3439,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Dia 356 de 365. Atos 9:17-18: Saulo voltou a ver. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 69 de 365. Atos 9:17-18: Saulo voltou a ver. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Dia 357 de 365. Lucas 5:5-6: Sobre a tua palavra, lançarei as redes. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 70 de 365. Lucas 5:5-6: Sobre a tua palavra, lançarei as redes. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -3525,7 +3525,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Dia 358 de 365. Oseias 6:3: Como a alva, a sua vinda é certa. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 71 de 365. Oseias 6:3: Como a alva, a sua vinda é certa. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Dia 359 de 365. Ageu 2:9: A glória desta última casa será maior. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 72 de 365. Ageu 2:9: A glória desta última casa será maior. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -3611,7 +3611,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Dia 360 de 365. Isaías 54:10: Os montes se retirarão. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 73 de 365. Isaías 54:10: Os montes se retirarão. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Dia 361 de 365. Salmos 30:11: Tornaste o meu pranto em dança. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 74 de 365. Salmos 30:11: Tornaste o meu pranto em dança. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Dia 362 de 365. 2 Pedro 3:9: O Senhor não retarda a promessa. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 75 de 365. 2 Pedro 3:9: O Senhor não retarda a promessa. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -3740,7 +3740,7 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Dia 363 de 365. Isaías 46:4: Até a velhice eu te carregarei. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 76 de 365. Isaías 46:4: Até a velhice eu te carregarei. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Dia 364 de 365. Números 6:24-26: O Senhor te abençoe e te guarde. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 77 de 365. Números 6:24-26: O Senhor te abençoe e te guarde. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -3826,7 +3826,7 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Dia 365 de 365. Judas 1:24-25: Àquele que é poderoso para vos guardar. #fe #recomeco #promessas #palavradodia</t>
+          <t>Dia 78 de 365. Judas 1:24-25: Àquele que é poderoso para vos guardar. #fe #recomeco #promessas #palavradodia</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Dia 1 de 365. Filipenses 4:6-7: Se a ansiedade te acordou hoje, ouça isso antes de começar o dia. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 79 de 365. Filipenses 4:6-7: Se a ansiedade te acordou hoje, ouça isso antes de começar o dia. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Dia 2 de 365. Mateus 6:34: Você está sofrendo hoje por algo que ainda nem aconteceu? #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 80 de 365. Mateus 6:34: Você está sofrendo hoje por algo que ainda nem aconteceu? #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -3955,7 +3955,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Dia 3 de 365. 1 Pedro 5:7: Tem uma coisa que você não contou para ninguém. Deus já sabe. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 81 de 365. 1 Pedro 5:7: Tem uma coisa que você não contou para ninguém. Deus já sabe. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -3998,7 +3998,7 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Dia 4 de 365. João 14:27: A paz que o mundo vende acaba. Essa não. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 82 de 365. João 14:27: A paz que o mundo vende acaba. Essa não. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -4041,7 +4041,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Dia 5 de 365. Salmos 94:19: Quando os pensamentos não param, leia isso. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 83 de 365. Salmos 94:19: Quando os pensamentos não param, leia isso. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -4084,7 +4084,7 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Dia 6 de 365. Isaías 26:3: Existe um tipo de paz que só vem de um lugar. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 84 de 365. Isaías 26:3: Existe um tipo de paz que só vem de um lugar. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Dia 7 de 365. Salmos 46:10: Às vezes a resposta é parar. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 85 de 365. Salmos 46:10: Às vezes a resposta é parar. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -4170,7 +4170,7 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Dia 8 de 365. Mateus 11:28-30: Cansado de carregar tudo sozinho? #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 86 de 365. Mateus 11:28-30: Cansado de carregar tudo sozinho? #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
@@ -4213,7 +4213,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Dia 9 de 365. Salmos 55:22: O que você está carregando que não é seu para carregar? #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 87 de 365. Salmos 55:22: O que você está carregando que não é seu para carregar? #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -4256,7 +4256,7 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Dia 10 de 365. Provérbios 12:25: Uma palavra boa muda o dia de alguém. Inclusive o seu. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 88 de 365. Provérbios 12:25: Uma palavra boa muda o dia de alguém. Inclusive o seu. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -4299,7 +4299,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Dia 11 de 365. Salmos 4:8: Para quem não consegue dormir de preocupação. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 89 de 365. Salmos 4:8: Para quem não consegue dormir de preocupação. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -4342,7 +4342,7 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Dia 12 de 365. Isaías 41:10: Se o medo de hoje parece maior que você, ouça isso. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 90 de 365. Isaías 41:10: Se o medo de hoje parece maior que você, ouça isso. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -4385,7 +4385,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Dia 13 de 365. Salmos 23:1-3: O salmo que milhões repetem quando a vida aperta. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 91 de 365. Salmos 23:1-3: O salmo que milhões repetem quando a vida aperta. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Dia 14 de 365. Romanos 8:28: Nem tudo que acontece é bom. Mas veja o que este versículo diz. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 92 de 365. Romanos 8:28: Nem tudo que acontece é bom. Mas veja o que este versículo diz. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -4471,7 +4471,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Dia 15 de 365. 2 Timóteo 1:7: O medo não veio de Deus. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 93 de 365. 2 Timóteo 1:7: O medo não veio de Deus. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Nova contagem, gancho e CTA: mais dias
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Eevu1kG1RwxjevYg68LqvH
</commit_message>
<xml_diff>
--- a/legendas-365.xlsx
+++ b/legendas-365.xlsx
@@ -4514,7 +4514,7 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Dia 16 de 365. Salmos 34:4: Busquei, e Ele respondeu. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 94 de 365. Salmos 34:4: Busquei, e Ele respondeu. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -4557,7 +4557,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Dia 17 de 365. Salmos 61:2: Quando o coração desfalece, para onde você corre? #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 95 de 365. Salmos 61:2: Quando o coração desfalece, para onde você corre? #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -4600,7 +4600,7 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Dia 18 de 365. Filipenses 4:8: Mude o que você alimenta na mente e o dia muda. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 96 de 365. Filipenses 4:8: Mude o que você alimenta na mente e o dia muda. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Dia 19 de 365. Salmos 139:23-24: Uma oração para quem está com o coração inquieto. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 97 de 365. Salmos 139:23-24: Uma oração para quem está com o coração inquieto. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -4686,7 +4686,7 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Dia 20 de 365. Lucas 12:25-26: Preocupação já resolveu algum problema seu? #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 98 de 365. Lucas 12:25-26: Preocupação já resolveu algum problema seu? #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
@@ -4729,7 +4729,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Dia 21 de 365. Josué 1:9: Uma ordem e uma promessa no mesmo versículo. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 99 de 365. Josué 1:9: Uma ordem e uma promessa no mesmo versículo. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -4772,7 +4772,7 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Dia 22 de 365. Salmos 121:1-2: De onde vem o seu socorro? #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 100 de 365. Salmos 121:1-2: De onde vem o seu socorro? #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
@@ -4815,7 +4815,7 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Dia 23 de 365. Isaías 40:31: Para quem está sem forças para continuar. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 101 de 365. Isaías 40:31: Para quem está sem forças para continuar. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -4858,7 +4858,7 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Dia 24 de 365. Êxodo 14:14: Tem batalhas que não são suas para lutar. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 102 de 365. Êxodo 14:14: Tem batalhas que não são suas para lutar. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
@@ -4901,7 +4901,7 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Dia 25 de 365. Salmos 56:3: Uma frase curta para repetir quando o medo chegar. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 103 de 365. Salmos 56:3: Uma frase curta para repetir quando o medo chegar. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>Dia 26 de 365. Mateus 6:26: Olhe os pássaros lá fora. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 104 de 365. Mateus 6:26: Olhe os pássaros lá fora. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
@@ -4987,7 +4987,7 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Dia 27 de 365. Salmos 3:3: Quando você está de cabeça baixa. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 105 de 365. Salmos 3:3: Quando você está de cabeça baixa. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -5030,7 +5030,7 @@
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Dia 28 de 365. Sofonias 3:17: Deus se alegra com você. Já pensou nisso? #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 106 de 365. Sofonias 3:17: Deus se alegra com você. Já pensou nisso? #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
@@ -5073,7 +5073,7 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Dia 29 de 365. João 16:33: Jesus nunca prometeu uma vida sem problemas. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 107 de 365. João 16:33: Jesus nunca prometeu uma vida sem problemas. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -5116,7 +5116,7 @@
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>Dia 30 de 365. Salmos 16:8: O segredo de quem não é abalado. #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 108 de 365. Salmos 16:8: O segredo de quem não é abalado. #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
@@ -5159,7 +5159,7 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Dia 31 de 365. Salmos 27:1: Se Deus é sua luz, de quem você vai ter medo? #fe #ansiedade #paz #palavradodia</t>
+          <t>Dia 109 de 365. Salmos 27:1: Se Deus é sua luz, de quem você vai ter medo? #fe #ansiedade #paz #palavradodia</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Dia 32 de 365. Deuteronômio 31:6: Você não vai enfrentar isso sozinho. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 110 de 365. Deuteronômio 31:6: Você não vai enfrentar isso sozinho. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
@@ -5245,7 +5245,7 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>Dia 33 de 365. Salmos 118:6: Uma pergunta para quem tem medo do que os outros vão fazer. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 111 de 365. Salmos 118:6: Uma pergunta para quem tem medo do que os outros vão fazer. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
@@ -5288,7 +5288,7 @@
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>Dia 34 de 365. Isaías 43:1-2: Você passou pelas águas e não se afogou. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 112 de 365. Isaías 43:1-2: Você passou pelas águas e não se afogou. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>Dia 35 de 365. Salmos 23:4: Para quem está atravessando um vale escuro. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 113 de 365. Salmos 23:4: Para quem está atravessando um vale escuro. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -5374,7 +5374,7 @@
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>Dia 36 de 365. Romanos 8:31: Se Deus é por você, quem será contra? #fe #coragem #medo #palavradodia</t>
+          <t>Dia 114 de 365. Romanos 8:31: Se Deus é por você, quem será contra? #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
@@ -5417,7 +5417,7 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>Dia 37 de 365. Hebreus 13:6: Diga em voz alta: o Senhor é o meu ajudador. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 115 de 365. Hebreus 13:6: Diga em voz alta: o Senhor é o meu ajudador. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
@@ -5460,7 +5460,7 @@
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>Dia 38 de 365. Provérbios 28:1: Por que algumas pessoas parecem não ter medo? #fe #coragem #medo #palavradodia</t>
+          <t>Dia 116 de 365. Provérbios 28:1: Por que algumas pessoas parecem não ter medo? #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
@@ -5503,7 +5503,7 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>Dia 39 de 365. Salmos 91:1-2: O salmo da proteção. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 117 de 365. Salmos 91:1-2: O salmo da proteção. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -5546,7 +5546,7 @@
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>Dia 40 de 365. Josué 1:7: Coragem para fazer o certo, não só o fácil. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 118 de 365. Josué 1:7: Coragem para fazer o certo, não só o fácil. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
@@ -5589,7 +5589,7 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>Dia 41 de 365. 1 Samuel 17:45: Davi diante do gigante. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 119 de 365. 1 Samuel 17:45: Davi diante do gigante. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -5632,7 +5632,7 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>Dia 42 de 365. Salmos 27:14: Coragem também é saber esperar. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 120 de 365. Salmos 27:14: Coragem também é saber esperar. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
@@ -5675,7 +5675,7 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>Dia 43 de 365. Isaías 12:2: Confiar sem medo. Dá para treinar isso? #fe #coragem #medo #palavradodia</t>
+          <t>Dia 121 de 365. Isaías 12:2: Confiar sem medo. Dá para treinar isso? #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -5718,7 +5718,7 @@
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>Dia 44 de 365. 2 Crônicas 20:15: A batalha não é sua. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 122 de 365. 2 Crônicas 20:15: A batalha não é sua. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
@@ -5761,7 +5761,7 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>Dia 45 de 365. Salmos 46:1-2: Mesmo que tudo desabe. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 123 de 365. Salmos 46:1-2: Mesmo que tudo desabe. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>Dia 46 de 365. Marcos 4:39-40: Jesus dormia no meio da tempestade. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 124 de 365. Marcos 4:39-40: Jesus dormia no meio da tempestade. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
@@ -5847,7 +5847,7 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>Dia 47 de 365. Mateus 14:29-31: Pedro andou sobre as águas. Até olhar para o vento. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 125 de 365. Mateus 14:29-31: Pedro andou sobre as águas. Até olhar para o vento. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -5890,7 +5890,7 @@
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>Dia 48 de 365. Salmos 112:7: Medo de notícia ruim? #fe #coragem #medo #palavradodia</t>
+          <t>Dia 126 de 365. Salmos 112:7: Medo de notícia ruim? #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>Dia 49 de 365. Lucas 1:37: Para quem acha que é tarde demais. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 127 de 365. Lucas 1:37: Para quem acha que é tarde demais. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -5976,7 +5976,7 @@
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>Dia 50 de 365. Juízes 6:12: Deus chamou de valente um homem escondido. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 128 de 365. Juízes 6:12: Deus chamou de valente um homem escondido. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>Dia 51 de 365. Salmos 31:24: Uma palavra para todos que esperam no Senhor. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 129 de 365. Salmos 31:24: Uma palavra para todos que esperam no Senhor. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
@@ -6062,7 +6062,7 @@
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>Dia 52 de 365. Ester 4:14: Talvez você esteja exatamente onde precisa estar. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 130 de 365. Ester 4:14: Talvez você esteja exatamente onde precisa estar. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
@@ -6105,7 +6105,7 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>Dia 53 de 365. Daniel 3:17-18: Fé que não depende do resultado. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 131 de 365. Daniel 3:17-18: Fé que não depende do resultado. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>Dia 54 de 365. Atos 18:9-10: Não se cale. Eu estou com você. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 132 de 365. Atos 18:9-10: Não se cale. Eu estou com você. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E133" s="2" t="inlineStr">
@@ -6191,7 +6191,7 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>Dia 55 de 365. Salmos 138:3: Ele respondeu no dia em que você clamou. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 133 de 365. Salmos 138:3: Ele respondeu no dia em que você clamou. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
@@ -6234,7 +6234,7 @@
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>Dia 56 de 365. Isaías 54:17: Nenhuma arma forjada contra você prosperará. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 134 de 365. Isaías 54:17: Nenhuma arma forjada contra você prosperará. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
@@ -6277,7 +6277,7 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>Dia 57 de 365. Provérbios 3:25-26: Não tema o pavor repentino. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 135 de 365. Provérbios 3:25-26: Não tema o pavor repentino. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
@@ -6320,7 +6320,7 @@
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>Dia 58 de 365. Neemias 4:14: Lembre-se de quem é o Senhor. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 136 de 365. Neemias 4:14: Lembre-se de quem é o Senhor. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr">
@@ -6363,7 +6363,7 @@
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>Dia 59 de 365. 2 Coríntios 12:9-10: Quando você é fraco, aí é que é forte. #fe #coragem #medo #palavradodia</t>
+          <t>Dia 137 de 365. 2 Coríntios 12:9-10: Quando você é fraco, aí é que é forte. #fe #coragem #medo #palavradodia</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>Dia 60 de 365. Lamentações 3:22-23: As misericórdias se renovam toda manhã. Inclusive nesta. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 138 de 365. Lamentações 3:22-23: As misericórdias se renovam toda manhã. Inclusive nesta. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E139" s="2" t="inlineStr">
@@ -6449,7 +6449,7 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>Dia 61 de 365. Jeremias 29:11: Deus tem planos para você. Bons. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 139 de 365. Jeremias 29:11: Deus tem planos para você. Bons. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
@@ -6492,7 +6492,7 @@
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>Dia 62 de 365. Romanos 15:13: Uma bênção para quem perdeu a esperança. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 140 de 365. Romanos 15:13: Uma bênção para quem perdeu a esperança. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E141" s="2" t="inlineStr">
@@ -6535,7 +6535,7 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>Dia 63 de 365. Salmos 42:11: Por que estás abatida, ó minha alma? #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 141 de 365. Salmos 42:11: Por que estás abatida, ó minha alma? #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
@@ -6578,7 +6578,7 @@
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>Dia 64 de 365. Isaías 43:19: Deus está fazendo algo novo. Você não percebe? #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 142 de 365. Isaías 43:19: Deus está fazendo algo novo. Você não percebe? #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>Dia 65 de 365. Romanos 5:3-5: A dor não é o fim da história. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 143 de 365. Romanos 5:3-5: A dor não é o fim da história. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="D145" s="2" t="inlineStr">
         <is>
-          <t>Dia 66 de 365. 2 Coríntios 4:16-18: Por fora você cansa. Por dentro, algo se renova. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 144 de 365. 2 Coríntios 4:16-18: Por fora você cansa. Por dentro, algo se renova. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E145" s="2" t="inlineStr">
@@ -6707,7 +6707,7 @@
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>Dia 67 de 365. Salmos 30:5: O choro pode durar uma noite. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 145 de 365. Salmos 30:5: O choro pode durar uma noite. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
@@ -6750,7 +6750,7 @@
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>Dia 68 de 365. Habacuque 3:17-18: Mesmo que nada dê certo. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 146 de 365. Habacuque 3:17-18: Mesmo que nada dê certo. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E147" s="2" t="inlineStr">
@@ -6793,7 +6793,7 @@
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>Dia 69 de 365. Hebreus 6:19: Uma âncora para a alma. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 147 de 365. Hebreus 6:19: Uma âncora para a alma. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
@@ -6836,7 +6836,7 @@
       </c>
       <c r="D149" s="2" t="inlineStr">
         <is>
-          <t>Dia 70 de 365. Salmos 40:1-2: Esperei com paciência. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 148 de 365. Salmos 40:1-2: Esperei com paciência. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E149" s="2" t="inlineStr">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>Dia 71 de 365. Isaías 61:3: Coroa em vez de cinzas. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 149 de 365. Isaías 61:3: Coroa em vez de cinzas. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
@@ -6922,7 +6922,7 @@
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>Dia 72 de 365. Romanos 8:18: O que vem é maior do que o que dói. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 150 de 365. Romanos 8:18: O que vem é maior do que o que dói. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
@@ -6965,7 +6965,7 @@
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>Dia 73 de 365. Miqueias 7:8: Caí, mas vou me levantar. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 151 de 365. Miqueias 7:8: Caí, mas vou me levantar. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>Dia 74 de 365. Salmos 147:3: Para quem está de coração partido. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 152 de 365. Salmos 147:3: Para quem está de coração partido. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
@@ -7051,7 +7051,7 @@
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>Dia 75 de 365. Joel 2:25: Deus pode restituir os anos perdidos. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 153 de 365. Joel 2:25: Deus pode restituir os anos perdidos. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
@@ -7094,7 +7094,7 @@
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>Dia 76 de 365. Jó 42:10: A história de Jó não termina na perda. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 154 de 365. Jó 42:10: A história de Jó não termina na perda. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr">
@@ -7137,7 +7137,7 @@
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>Dia 77 de 365. Salmos 34:18: Deus está perto. Especialmente agora. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 155 de 365. Salmos 34:18: Deus está perto. Especialmente agora. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
@@ -7180,7 +7180,7 @@
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>Dia 78 de 365. Apocalipse 21:4: Um dia sem lágrimas. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 156 de 365. Apocalipse 21:4: Um dia sem lágrimas. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr">
@@ -7223,7 +7223,7 @@
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>Dia 79 de 365. Romanos 12:12: Três atitudes para dias difíceis. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 157 de 365. Romanos 12:12: Três atitudes para dias difíceis. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
@@ -7266,7 +7266,7 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>Dia 80 de 365. Isaías 40:29: Ele dá força ao cansado. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 158 de 365. Isaías 40:29: Ele dá força ao cansado. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
@@ -7309,7 +7309,7 @@
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>Dia 81 de 365. Salmos 71:20: Você vai voltar a viver. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 159 de 365. Salmos 71:20: Você vai voltar a viver. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
@@ -7352,7 +7352,7 @@
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>Dia 82 de 365. 1 Pedro 1:3: Uma esperança viva. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 160 de 365. 1 Pedro 1:3: Uma esperança viva. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
@@ -7395,7 +7395,7 @@
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>Dia 83 de 365. Gênesis 50:20: O mal que planejaram contra você. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 161 de 365. Gênesis 50:20: O mal que planejaram contra você. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
@@ -7438,7 +7438,7 @@
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>Dia 84 de 365. Salmos 126:5-6: Quem semeia com lágrimas. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 162 de 365. Salmos 126:5-6: Quem semeia com lágrimas. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
@@ -7481,7 +7481,7 @@
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>Dia 85 de 365. Isaías 9:2: Uma luz no meio da escuridão. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 163 de 365. Isaías 9:2: Uma luz no meio da escuridão. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E164" s="2" t="inlineStr">
@@ -7524,7 +7524,7 @@
       </c>
       <c r="D165" s="2" t="inlineStr">
         <is>
-          <t>Dia 86 de 365. Salmos 62:5: Descanse, ó minha alma. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 164 de 365. Salmos 62:5: Descanse, ó minha alma. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E165" s="2" t="inlineStr">
@@ -7567,7 +7567,7 @@
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>Dia 87 de 365. Isaías 35:3-4: Fortalecei as mãos fracas. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 165 de 365. Isaías 35:3-4: Fortalecei as mãos fracas. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E166" s="2" t="inlineStr">
@@ -7610,7 +7610,7 @@
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>Dia 88 de 365. 2 Coríntios 4:8-9: Apertado, mas não esmagado. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 166 de 365. 2 Coríntios 4:8-9: Apertado, mas não esmagado. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E167" s="2" t="inlineStr">
@@ -7653,7 +7653,7 @@
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>Dia 89 de 365. Salmos 33:20-22: Nossa alma espera no Senhor. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 167 de 365. Salmos 33:20-22: Nossa alma espera no Senhor. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E168" s="2" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>Dia 90 de 365. Mateus 28:20: Até o fim. Todos os dias. #fe #esperanca #forca #palavradodia</t>
+          <t>Dia 168 de 365. Mateus 28:20: Até o fim. Todos os dias. #fe #esperanca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E169" s="2" t="inlineStr">
@@ -7739,7 +7739,7 @@
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>Dia 91 de 365. Efésios 4:32: Perdoar não é dizer que não doeu. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 169 de 365. Efésios 4:32: Perdoar não é dizer que não doeu. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E170" s="2" t="inlineStr">
@@ -7782,7 +7782,7 @@
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>Dia 92 de 365. Colossenses 3:13: Tem alguém que você ainda não perdoou? #fe #perdao #graca #palavradodia</t>
+          <t>Dia 170 de 365. Colossenses 3:13: Tem alguém que você ainda não perdoou? #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E171" s="2" t="inlineStr">
@@ -7868,7 +7868,7 @@
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>Dia 94 de 365. Mateus 18:21-22: Quantas vezes eu tenho que perdoar? #fe #perdao #graca #palavradodia</t>
+          <t>Dia 172 de 365. Mateus 18:21-22: Quantas vezes eu tenho que perdoar? #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E173" s="2" t="inlineStr">
@@ -7911,7 +7911,7 @@
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>Dia 95 de 365. 1 João 1:9: Para quem acha que errou demais. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 173 de 365. 1 João 1:9: Para quem acha que errou demais. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E174" s="2" t="inlineStr">
@@ -7954,7 +7954,7 @@
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>Dia 96 de 365. Salmos 103:12: Até onde Deus jogou os seus erros? #fe #perdao #graca #palavradodia</t>
+          <t>Dia 174 de 365. Salmos 103:12: Até onde Deus jogou os seus erros? #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E175" s="2" t="inlineStr">
@@ -7997,7 +7997,7 @@
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>Dia 97 de 365. Isaías 1:18: Ainda que seus pecados sejam como escarlate. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 175 de 365. Isaías 1:18: Ainda que seus pecados sejam como escarlate. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E176" s="2" t="inlineStr">
@@ -8040,7 +8040,7 @@
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>Dia 98 de 365. Lucas 15:20: O pai correu. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 176 de 365. Lucas 15:20: O pai correu. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E177" s="2" t="inlineStr">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>Dia 99 de 365. Lucas 23:34: Jesus perdoou enquanto ainda doía. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 177 de 365. Lucas 23:34: Jesus perdoou enquanto ainda doía. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
@@ -8126,7 +8126,7 @@
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>Dia 100 de 365. Miqueias 7:18-19: Deus lança os pecados no fundo do mar. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 178 de 365. Miqueias 7:18-19: Deus lança os pecados no fundo do mar. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E179" s="2" t="inlineStr">
@@ -8169,7 +8169,7 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>Dia 101 de 365. Romanos 12:17-19: Não pague o mal com mal. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 179 de 365. Romanos 12:17-19: Não pague o mal com mal. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
@@ -8212,7 +8212,7 @@
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>Dia 102 de 365. Salmos 32:1-2: Feliz é quem foi perdoado. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 180 de 365. Salmos 32:1-2: Feliz é quem foi perdoado. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E181" s="2" t="inlineStr">
@@ -8255,7 +8255,7 @@
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>Dia 103 de 365. Marcos 11:25: Antes de orar, solte. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 181 de 365. Marcos 11:25: Antes de orar, solte. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr">
@@ -8298,7 +8298,7 @@
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>Dia 104 de 365. Hebreus 8:12: Deus decide esquecer. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 182 de 365. Hebreus 8:12: Deus decide esquecer. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E183" s="2" t="inlineStr">
@@ -8341,7 +8341,7 @@
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>Dia 105 de 365. Gênesis 45:4-5: José perdoou os irmãos que o venderam. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 183 de 365. Gênesis 45:4-5: José perdoou os irmãos que o venderam. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr">
@@ -8384,7 +8384,7 @@
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>Dia 106 de 365. Provérbios 19:11: Saber deixar passar é sabedoria. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 184 de 365. Provérbios 19:11: Saber deixar passar é sabedoria. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E185" s="2" t="inlineStr">
@@ -8427,7 +8427,7 @@
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>Dia 107 de 365. 2 Coríntios 5:17: Você não é mais quem era. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 185 de 365. 2 Coríntios 5:17: Você não é mais quem era. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E186" s="2" t="inlineStr">
@@ -8470,7 +8470,7 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>Dia 108 de 365. Romanos 8:1: Nenhuma condenação. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 186 de 365. Romanos 8:1: Nenhuma condenação. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E187" s="2" t="inlineStr">
@@ -8513,7 +8513,7 @@
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>Dia 109 de 365. Lucas 6:37: Não julgue, e não será julgado. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 187 de 365. Lucas 6:37: Não julgue, e não será julgado. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E188" s="2" t="inlineStr">
@@ -8556,7 +8556,7 @@
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>Dia 110 de 365. Salmos 51:10: Uma oração para recomeçar por dentro. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 188 de 365. Salmos 51:10: Uma oração para recomeçar por dentro. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E189" s="2" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>Dia 111 de 365. Atos 3:19: Arrepender e ser renovado. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 189 de 365. Atos 3:19: Arrepender e ser renovado. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E190" s="2" t="inlineStr">
@@ -8642,7 +8642,7 @@
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>Dia 112 de 365. Mateus 5:23-24: Antes da oferta, a reconciliação. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 190 de 365. Mateus 5:23-24: Antes da oferta, a reconciliação. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E191" s="2" t="inlineStr">
@@ -8685,7 +8685,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>Dia 113 de 365. Efésios 4:26-27: Não deixe o sol se pôr sobre a sua ira. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 191 de 365. Efésios 4:26-27: Não deixe o sol se pôr sobre a sua ira. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E192" s="2" t="inlineStr">
@@ -8728,7 +8728,7 @@
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>Dia 114 de 365. Lucas 7:47: Quem foi muito perdoado, ama muito. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 192 de 365. Lucas 7:47: Quem foi muito perdoado, ama muito. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E193" s="2" t="inlineStr">
@@ -8771,7 +8771,7 @@
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>Dia 115 de 365. João 8:10-11: Nem eu te condeno. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 193 de 365. João 8:10-11: Nem eu te condeno. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E194" s="2" t="inlineStr">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>Dia 116 de 365. Isaías 43:25: Deus apaga por amor a si mesmo. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 194 de 365. Isaías 43:25: Deus apaga por amor a si mesmo. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E195" s="2" t="inlineStr">
@@ -8857,7 +8857,7 @@
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>Dia 117 de 365. Salmos 130:3-4: Se Deus guardasse a lista. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 195 de 365. Salmos 130:3-4: Se Deus guardasse a lista. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E196" s="2" t="inlineStr">
@@ -8900,7 +8900,7 @@
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>Dia 118 de 365. Colossenses 2:13-14: A dívida foi pregada na cruz. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 196 de 365. Colossenses 2:13-14: A dívida foi pregada na cruz. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E197" s="2" t="inlineStr">
@@ -8943,7 +8943,7 @@
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>Dia 119 de 365. 1 Pedro 3:9: Responda com bênção. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 197 de 365. 1 Pedro 3:9: Responda com bênção. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr">
@@ -8986,7 +8986,7 @@
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>Dia 120 de 365. Lucas 17:3-4: Perdoar também quando se repete. #fe #perdao #graca #palavradodia</t>
+          <t>Dia 198 de 365. Lucas 17:3-4: Perdoar também quando se repete. #fe #perdao #graca #palavradodia</t>
         </is>
       </c>
       <c r="E199" s="2" t="inlineStr">
@@ -9029,7 +9029,7 @@
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>Dia 121 de 365. Josué 24:15: Eu e a minha casa serviremos ao Senhor. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 199 de 365. Josué 24:15: Eu e a minha casa serviremos ao Senhor. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E200" s="2" t="inlineStr">
@@ -9072,7 +9072,7 @@
       </c>
       <c r="D201" s="2" t="inlineStr">
         <is>
-          <t>Dia 122 de 365. Salmos 127:1: Se o Senhor não edificar a casa. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 200 de 365. Salmos 127:1: Se o Senhor não edificar a casa. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E201" s="2" t="inlineStr">
@@ -9115,7 +9115,7 @@
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>Dia 123 de 365. Provérbios 22:6: Ensina a criança no caminho. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 201 de 365. Provérbios 22:6: Ensina a criança no caminho. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E202" s="2" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="D203" s="2" t="inlineStr">
         <is>
-          <t>Dia 124 de 365. Efésios 6:1-3: Honrar pai e mãe tem uma promessa. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 202 de 365. Efésios 6:1-3: Honrar pai e mãe tem uma promessa. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E203" s="2" t="inlineStr">
@@ -9201,7 +9201,7 @@
       </c>
       <c r="D204" s="2" t="inlineStr">
         <is>
-          <t>Dia 125 de 365. Eclesiastes 4:9-10: Dois são melhores que um. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 203 de 365. Eclesiastes 4:9-10: Dois são melhores que um. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E204" s="2" t="inlineStr">
@@ -9244,7 +9244,7 @@
       </c>
       <c r="D205" s="2" t="inlineStr">
         <is>
-          <t>Dia 126 de 365. Eclesiastes 4:12: O cordão de três dobras. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 204 de 365. Eclesiastes 4:12: O cordão de três dobras. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E205" s="2" t="inlineStr">
@@ -9287,7 +9287,7 @@
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>Dia 127 de 365. Rute 1:16-17: Aonde quer que fores, irei. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 205 de 365. Rute 1:16-17: Aonde quer que fores, irei. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E206" s="2" t="inlineStr">
@@ -9330,7 +9330,7 @@
       </c>
       <c r="D207" s="2" t="inlineStr">
         <is>
-          <t>Dia 128 de 365. Provérbios 17:17: O amigo ama em todo tempo. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 206 de 365. Provérbios 17:17: O amigo ama em todo tempo. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E207" s="2" t="inlineStr">
@@ -9373,7 +9373,7 @@
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>Dia 129 de 365. Colossenses 3:14: Acima de tudo, o amor. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 207 de 365. Colossenses 3:14: Acima de tudo, o amor. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E208" s="2" t="inlineStr">
@@ -9459,7 +9459,7 @@
       </c>
       <c r="D210" s="2" t="inlineStr">
         <is>
-          <t>Dia 131 de 365. Gênesis 2:24: Deixar e unir. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 209 de 365. Gênesis 2:24: Deixar e unir. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E210" s="2" t="inlineStr">
@@ -9502,7 +9502,7 @@
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>Dia 132 de 365. Provérbios 31:10-11: Quem achará uma mulher virtuosa? #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 210 de 365. Provérbios 31:10-11: Quem achará uma mulher virtuosa? #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E211" s="2" t="inlineStr">
@@ -9545,7 +9545,7 @@
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
-          <t>Dia 133 de 365. Efésios 5:25: Amar como Cristo amou a igreja. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 211 de 365. Efésios 5:25: Amar como Cristo amou a igreja. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E212" s="2" t="inlineStr">
@@ -9588,7 +9588,7 @@
       </c>
       <c r="D213" s="2" t="inlineStr">
         <is>
-          <t>Dia 134 de 365. Salmos 133:1: Como é bom viver em união. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 212 de 365. Salmos 133:1: Como é bom viver em união. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E213" s="2" t="inlineStr">
@@ -9631,7 +9631,7 @@
       </c>
       <c r="D214" s="2" t="inlineStr">
         <is>
-          <t>Dia 135 de 365. Provérbios 15:1: A resposta branda desvia o furor. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 213 de 365. Provérbios 15:1: A resposta branda desvia o furor. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E214" s="2" t="inlineStr">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="D215" s="2" t="inlineStr">
         <is>
-          <t>Dia 136 de 365. Tiago 1:19: Ouvir mais, falar menos. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 214 de 365. Tiago 1:19: Ouvir mais, falar menos. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E215" s="2" t="inlineStr">
@@ -9717,7 +9717,7 @@
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>Dia 137 de 365. 1 Pedro 4:8: O amor cobre muitos pecados. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 215 de 365. 1 Pedro 4:8: O amor cobre muitos pecados. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E216" s="2" t="inlineStr">
@@ -9760,7 +9760,7 @@
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>Dia 138 de 365. Malaquias 4:6: Corações que voltam. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 216 de 365. Malaquias 4:6: Corações que voltam. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E217" s="2" t="inlineStr">
@@ -9803,7 +9803,7 @@
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>Dia 139 de 365. Salmos 68:6: Deus faz o solitário habitar em família. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 217 de 365. Salmos 68:6: Deus faz o solitário habitar em família. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E218" s="2" t="inlineStr">
@@ -9846,7 +9846,7 @@
       </c>
       <c r="D219" s="2" t="inlineStr">
         <is>
-          <t>Dia 140 de 365. Provérbios 27:17: Ferro afia ferro. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 218 de 365. Provérbios 27:17: Ferro afia ferro. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E219" s="2" t="inlineStr">
@@ -9889,7 +9889,7 @@
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t>Dia 141 de 365. Romanos 12:10: Amai-vos cordialmente. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 219 de 365. Romanos 12:10: Amai-vos cordialmente. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E220" s="2" t="inlineStr">
@@ -9932,7 +9932,7 @@
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>Dia 142 de 365. 1 Tessalonicenses 5:11: Encorajem uns aos outros. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 220 de 365. 1 Tessalonicenses 5:11: Encorajem uns aos outros. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E221" s="2" t="inlineStr">
@@ -9975,7 +9975,7 @@
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>Dia 143 de 365. Lucas 2:51-52: Jesus também viveu em família. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 221 de 365. Lucas 2:51-52: Jesus também viveu em família. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E222" s="2" t="inlineStr">
@@ -10018,7 +10018,7 @@
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>Dia 144 de 365. Provérbios 18:24: Há amigo mais chegado que um irmão. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 222 de 365. Provérbios 18:24: Há amigo mais chegado que um irmão. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E223" s="2" t="inlineStr">
@@ -10061,7 +10061,7 @@
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>Dia 145 de 365. João 15:13: Maior amor não há. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 223 de 365. João 15:13: Maior amor não há. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E224" s="2" t="inlineStr">
@@ -10104,7 +10104,7 @@
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>Dia 146 de 365. Gálatas 6:2: Levai as cargas uns dos outros. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 224 de 365. Gálatas 6:2: Levai as cargas uns dos outros. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E225" s="2" t="inlineStr">
@@ -10147,7 +10147,7 @@
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>Dia 147 de 365. Filipenses 2:3-4: Considere os outros superiores a si mesmo. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 225 de 365. Filipenses 2:3-4: Considere os outros superiores a si mesmo. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E226" s="2" t="inlineStr">
@@ -10190,7 +10190,7 @@
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>Dia 148 de 365. Salmos 103:13: Como um pai se compadece dos filhos. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 226 de 365. Salmos 103:13: Como um pai se compadece dos filhos. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E227" s="2" t="inlineStr">
@@ -10233,7 +10233,7 @@
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>Dia 149 de 365. Isaías 49:15: Uma mãe pode esquecer o filho? #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 227 de 365. Isaías 49:15: Uma mãe pode esquecer o filho? #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E228" s="2" t="inlineStr">
@@ -10276,7 +10276,7 @@
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>Dia 150 de 365. 1 João 4:11: Se Deus nos amou assim. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 228 de 365. 1 João 4:11: Se Deus nos amou assim. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E229" s="2" t="inlineStr">
@@ -10319,7 +10319,7 @@
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>Dia 151 de 365. Hebreus 13:1: Permaneça o amor fraternal. #fe #familia #relacionamentos #palavradodia</t>
+          <t>Dia 229 de 365. Hebreus 13:1: Permaneça o amor fraternal. #fe #familia #relacionamentos #palavradodia</t>
         </is>
       </c>
       <c r="E230" s="2" t="inlineStr">
@@ -10362,7 +10362,7 @@
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>Dia 152 de 365. 1 Tessalonicenses 5:18: Em tudo dai graças. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 230 de 365. 1 Tessalonicenses 5:18: Em tudo dai graças. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E231" s="2" t="inlineStr">
@@ -10405,7 +10405,7 @@
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>Dia 153 de 365. Salmos 118:24: Este é o dia que o Senhor fez. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 231 de 365. Salmos 118:24: Este é o dia que o Senhor fez. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E232" s="2" t="inlineStr">
@@ -10448,7 +10448,7 @@
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>Dia 154 de 365. Salmos 100:4: Entre pelas portas com ação de graças. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 232 de 365. Salmos 100:4: Entre pelas portas com ação de graças. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E233" s="2" t="inlineStr">
@@ -10491,7 +10491,7 @@
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>Dia 155 de 365. Colossenses 3:15: E sede agradecidos. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 233 de 365. Colossenses 3:15: E sede agradecidos. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E234" s="2" t="inlineStr">
@@ -10534,7 +10534,7 @@
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>Dia 156 de 365. Salmos 103:2: Não te esqueças de nenhum dos seus benefícios. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 234 de 365. Salmos 103:2: Não te esqueças de nenhum dos seus benefícios. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E235" s="2" t="inlineStr">
@@ -10577,7 +10577,7 @@
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>Dia 157 de 365. Lucas 17:15-16: Dos dez curados, só um voltou para agradecer. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 235 de 365. Lucas 17:15-16: Dos dez curados, só um voltou para agradecer. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E236" s="2" t="inlineStr">
@@ -10620,7 +10620,7 @@
       </c>
       <c r="D237" s="2" t="inlineStr">
         <is>
-          <t>Dia 158 de 365. Tiago 1:17: Todo bem vem do alto. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 236 de 365. Tiago 1:17: Todo bem vem do alto. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E237" s="2" t="inlineStr">
@@ -10663,7 +10663,7 @@
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>Dia 159 de 365. Salmos 136:1: A misericórdia dEle dura para sempre. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 237 de 365. Salmos 136:1: A misericórdia dEle dura para sempre. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E238" s="2" t="inlineStr">
@@ -10706,7 +10706,7 @@
       </c>
       <c r="D239" s="2" t="inlineStr">
         <is>
-          <t>Dia 160 de 365. Filipenses 4:11-12: Aprendi a contentar-me. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 238 de 365. Filipenses 4:11-12: Aprendi a contentar-me. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E239" s="2" t="inlineStr">
@@ -10749,7 +10749,7 @@
       </c>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>Dia 161 de 365. Salmos 9:1: De todo o coração. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 239 de 365. Salmos 9:1: De todo o coração. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E240" s="2" t="inlineStr">
@@ -10792,7 +10792,7 @@
       </c>
       <c r="D241" s="2" t="inlineStr">
         <is>
-          <t>Dia 162 de 365. Salmos 107:1: Dai graças ao Senhor, porque Ele é bom. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 240 de 365. Salmos 107:1: Dai graças ao Senhor, porque Ele é bom. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E241" s="2" t="inlineStr">
@@ -10835,7 +10835,7 @@
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>Dia 163 de 365. Efésios 5:20: Dando sempre graças por tudo. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 241 de 365. Efésios 5:20: Dando sempre graças por tudo. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E242" s="2" t="inlineStr">
@@ -10878,7 +10878,7 @@
       </c>
       <c r="D243" s="2" t="inlineStr">
         <is>
-          <t>Dia 164 de 365. Hebreus 12:28: Um reino que não pode ser abalado. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 242 de 365. Hebreus 12:28: Um reino que não pode ser abalado. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E243" s="2" t="inlineStr">
@@ -10921,7 +10921,7 @@
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>Dia 165 de 365. Salmos 92:1-2: Bom é render graças de manhã e de noite. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 243 de 365. Salmos 92:1-2: Bom é render graças de manhã e de noite. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E244" s="2" t="inlineStr">
@@ -10964,7 +10964,7 @@
       </c>
       <c r="D245" s="2" t="inlineStr">
         <is>
-          <t>Dia 166 de 365. 1 Crônicas 16:34: Rendei graças ao Senhor. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 244 de 365. 1 Crônicas 16:34: Rendei graças ao Senhor. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E245" s="2" t="inlineStr">
@@ -11007,7 +11007,7 @@
       </c>
       <c r="D246" s="2" t="inlineStr">
         <is>
-          <t>Dia 167 de 365. 2 Coríntios 9:15: Graças a Deus pelo seu dom inefável. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 245 de 365. 2 Coríntios 9:15: Graças a Deus pelo seu dom inefável. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E246" s="2" t="inlineStr">
@@ -11050,7 +11050,7 @@
       </c>
       <c r="D247" s="2" t="inlineStr">
         <is>
-          <t>Dia 168 de 365. Salmos 34:1: Bendirei o Senhor em todo o tempo. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 246 de 365. Salmos 34:1: Bendirei o Senhor em todo o tempo. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E247" s="2" t="inlineStr">
@@ -11093,7 +11093,7 @@
       </c>
       <c r="D248" s="2" t="inlineStr">
         <is>
-          <t>Dia 169 de 365. Daniel 6:10: Daniel orava e dava graças três vezes ao dia. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 247 de 365. Daniel 6:10: Daniel orava e dava graças três vezes ao dia. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E248" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Nova contagem, gancho e CTA nos dias restantes
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Eevu1kG1RwxjevYg68LqvH
</commit_message>
<xml_diff>
--- a/legendas-365.xlsx
+++ b/legendas-365.xlsx
@@ -515,7 +515,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Dia 288 de 365. Salmos 36:7: Quão preciosa é a tua benignidade. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 1 de 365. Salmos 36:7: Quão preciosa é a tua benignidade. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Dia 289 de 365. Salmos 63:3: O teu amor é melhor do que a vida. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 2 de 365. Salmos 63:3: O teu amor é melhor do que a vida. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Dia 290 de 365. Cantares 8:7: As muitas águas não podem apagar o amor. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 3 de 365. Cantares 8:7: As muitas águas não podem apagar o amor. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Dia 291 de 365. Lucas 10:33-34: O bom samaritano parou. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 4 de 365. Lucas 10:33-34: O bom samaritano parou. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Dia 293 de 365. Gálatas 5:13-14: Sirvam uns aos outros pelo amor. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 6 de 365. Gálatas 5:13-14: Sirvam uns aos outros pelo amor. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -11136,7 +11136,7 @@
       </c>
       <c r="D249" s="2" t="inlineStr">
         <is>
-          <t>Dia 170 de 365. Salmos 50:23: A gratidão honra a Deus. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 248 de 365. Salmos 50:23: A gratidão honra a Deus. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E249" s="2" t="inlineStr">
@@ -11179,7 +11179,7 @@
       </c>
       <c r="D250" s="2" t="inlineStr">
         <is>
-          <t>Dia 171 de 365. Romanos 1:21: O perigo de esquecer de agradecer. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 249 de 365. Romanos 1:21: O perigo de esquecer de agradecer. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E250" s="2" t="inlineStr">
@@ -11222,7 +11222,7 @@
       </c>
       <c r="D251" s="2" t="inlineStr">
         <is>
-          <t>Dia 172 de 365. Salmos 16:6: As cordas caíram em lugares deliciosos. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 250 de 365. Salmos 16:6: As cordas caíram em lugares deliciosos. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E251" s="2" t="inlineStr">
@@ -11265,7 +11265,7 @@
       </c>
       <c r="D252" s="2" t="inlineStr">
         <is>
-          <t>Dia 173 de 365. Salmos 145:9: O Senhor é bom para todos. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 251 de 365. Salmos 145:9: O Senhor é bom para todos. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E252" s="2" t="inlineStr">
@@ -11308,7 +11308,7 @@
       </c>
       <c r="D253" s="2" t="inlineStr">
         <is>
-          <t>Dia 174 de 365. João 6:11: Jesus deu graças antes do milagre. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 252 de 365. João 6:11: Jesus deu graças antes do milagre. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E253" s="2" t="inlineStr">
@@ -11351,7 +11351,7 @@
       </c>
       <c r="D254" s="2" t="inlineStr">
         <is>
-          <t>Dia 175 de 365. Salmos 95:2: Cheguemos com ações de graças. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 253 de 365. Salmos 95:2: Cheguemos com ações de graças. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E254" s="2" t="inlineStr">
@@ -11394,7 +11394,7 @@
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>Dia 176 de 365. Lamentações 3:24: A minha porção é o Senhor. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 254 de 365. Lamentações 3:24: A minha porção é o Senhor. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E255" s="2" t="inlineStr">
@@ -11437,7 +11437,7 @@
       </c>
       <c r="D256" s="2" t="inlineStr">
         <is>
-          <t>Dia 177 de 365. Salmos 116:12: Que darei ao Senhor por todos os benefícios? #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 255 de 365. Salmos 116:12: Que darei ao Senhor por todos os benefícios? #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E256" s="2" t="inlineStr">
@@ -11480,7 +11480,7 @@
       </c>
       <c r="D257" s="2" t="inlineStr">
         <is>
-          <t>Dia 178 de 365. Atos 16:25: Paulo e Silas cantavam presos. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 256 de 365. Atos 16:25: Paulo e Silas cantavam presos. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E257" s="2" t="inlineStr">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="D258" s="2" t="inlineStr">
         <is>
-          <t>Dia 179 de 365. Salmos 103:3-5: Ele perdoa, sara, resgata, coroa, farta. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 257 de 365. Salmos 103:3-5: Ele perdoa, sara, resgata, coroa, farta. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E258" s="2" t="inlineStr">
@@ -11566,7 +11566,7 @@
       </c>
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>Dia 180 de 365. Salmos 65:11: Coroas o ano com a tua bondade. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 258 de 365. Salmos 65:11: Coroas o ano com a tua bondade. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E259" s="2" t="inlineStr">
@@ -11609,7 +11609,7 @@
       </c>
       <c r="D260" s="2" t="inlineStr">
         <is>
-          <t>Dia 181 de 365. Neemias 8:10: A alegria do Senhor é a vossa força. #fe #gratidao #louvor #palavradodia</t>
+          <t>Dia 259 de 365. Neemias 8:10: A alegria do Senhor é a vossa força. #fe #gratidao #louvor #palavradodia</t>
         </is>
       </c>
       <c r="E260" s="2" t="inlineStr">
@@ -11652,7 +11652,7 @@
       </c>
       <c r="D261" s="2" t="inlineStr">
         <is>
-          <t>Dia 182 de 365. Colossenses 3:23: Trabalhe como se fosse para Deus. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 260 de 365. Colossenses 3:23: Trabalhe como se fosse para Deus. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E261" s="2" t="inlineStr">
@@ -11695,7 +11695,7 @@
       </c>
       <c r="D262" s="2" t="inlineStr">
         <is>
-          <t>Dia 183 de 365. Provérbios 16:3: Entregue ao Senhor as suas obras. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 261 de 365. Provérbios 16:3: Entregue ao Senhor as suas obras. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E262" s="2" t="inlineStr">
@@ -11738,7 +11738,7 @@
       </c>
       <c r="D263" s="2" t="inlineStr">
         <is>
-          <t>Dia 184 de 365. Efésios 2:10: Você foi feito com propósito. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 262 de 365. Efésios 2:10: Você foi feito com propósito. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E263" s="2" t="inlineStr">
@@ -11781,7 +11781,7 @@
       </c>
       <c r="D264" s="2" t="inlineStr">
         <is>
-          <t>Dia 185 de 365. Jeremias 1:5: Antes de te formar, eu te conheci. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 263 de 365. Jeremias 1:5: Antes de te formar, eu te conheci. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E264" s="2" t="inlineStr">
@@ -11824,7 +11824,7 @@
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
-          <t>Dia 186 de 365. Provérbios 14:23: Em todo trabalho há proveito. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 264 de 365. Provérbios 14:23: Em todo trabalho há proveito. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E265" s="2" t="inlineStr">
@@ -11867,7 +11867,7 @@
       </c>
       <c r="D266" s="2" t="inlineStr">
         <is>
-          <t>Dia 187 de 365. Eclesiastes 9:10: Faça com todas as suas forças. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 265 de 365. Eclesiastes 9:10: Faça com todas as suas forças. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E266" s="2" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="D267" s="2" t="inlineStr">
         <is>
-          <t>Dia 188 de 365. Provérbios 22:29: O diligente servirá diante de reis. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 266 de 365. Provérbios 22:29: O diligente servirá diante de reis. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E267" s="2" t="inlineStr">
@@ -11953,7 +11953,7 @@
       </c>
       <c r="D268" s="2" t="inlineStr">
         <is>
-          <t>Dia 189 de 365. Filipenses 1:6: Deus termina o que começa. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 267 de 365. Filipenses 1:6: Deus termina o que começa. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E268" s="2" t="inlineStr">
@@ -11996,7 +11996,7 @@
       </c>
       <c r="D269" s="2" t="inlineStr">
         <is>
-          <t>Dia 190 de 365. Gálatas 6:9: Não se canse de fazer o bem. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 268 de 365. Gálatas 6:9: Não se canse de fazer o bem. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E269" s="2" t="inlineStr">
@@ -12039,7 +12039,7 @@
       </c>
       <c r="D270" s="2" t="inlineStr">
         <is>
-          <t>Dia 191 de 365. Salmos 90:17: Confirma a obra das nossas mãos. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 269 de 365. Salmos 90:17: Confirma a obra das nossas mãos. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E270" s="2" t="inlineStr">
@@ -12082,7 +12082,7 @@
       </c>
       <c r="D271" s="2" t="inlineStr">
         <is>
-          <t>Dia 192 de 365. Romanos 12:6-8: Cada um tem um dom diferente. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 270 de 365. Romanos 12:6-8: Cada um tem um dom diferente. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E271" s="2" t="inlineStr">
@@ -12125,7 +12125,7 @@
       </c>
       <c r="D272" s="2" t="inlineStr">
         <is>
-          <t>Dia 193 de 365. 1 Pedro 4:10: Seu dom é para servir. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 271 de 365. 1 Pedro 4:10: Seu dom é para servir. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E272" s="2" t="inlineStr">
@@ -12168,7 +12168,7 @@
       </c>
       <c r="D273" s="2" t="inlineStr">
         <is>
-          <t>Dia 194 de 365. Provérbios 6:6-8: Olhe para a formiga. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 272 de 365. Provérbios 6:6-8: Olhe para a formiga. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E273" s="2" t="inlineStr">
@@ -12211,7 +12211,7 @@
       </c>
       <c r="D274" s="2" t="inlineStr">
         <is>
-          <t>Dia 195 de 365. Mateus 25:21: Fiel no pouco. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 273 de 365. Mateus 25:21: Fiel no pouco. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E274" s="2" t="inlineStr">
@@ -12254,7 +12254,7 @@
       </c>
       <c r="D275" s="2" t="inlineStr">
         <is>
-          <t>Dia 196 de 365. Neemias 2:20: O Deus dos céus nos fará prosperar. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 274 de 365. Neemias 2:20: O Deus dos céus nos fará prosperar. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E275" s="2" t="inlineStr">
@@ -12297,7 +12297,7 @@
       </c>
       <c r="D276" s="2" t="inlineStr">
         <is>
-          <t>Dia 197 de 365. Provérbios 13:4: O desejo do preguiçoso não se realiza. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 275 de 365. Provérbios 13:4: O desejo do preguiçoso não se realiza. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E276" s="2" t="inlineStr">
@@ -12340,7 +12340,7 @@
       </c>
       <c r="D277" s="2" t="inlineStr">
         <is>
-          <t>Dia 198 de 365. Mateus 5:14-16: Você é a luz do mundo. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 276 de 365. Mateus 5:14-16: Você é a luz do mundo. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E277" s="2" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="D278" s="2" t="inlineStr">
         <is>
-          <t>Dia 199 de 365. 1 Coríntios 15:58: Seu trabalho no Senhor não é em vão. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 277 de 365. 1 Coríntios 15:58: Seu trabalho no Senhor não é em vão. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E278" s="2" t="inlineStr">
@@ -12426,7 +12426,7 @@
       </c>
       <c r="D279" s="2" t="inlineStr">
         <is>
-          <t>Dia 200 de 365. Deuteronômio 8:18: É Ele quem dá força para conquistar. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 278 de 365. Deuteronômio 8:18: É Ele quem dá força para conquistar. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E279" s="2" t="inlineStr">
@@ -12469,7 +12469,7 @@
       </c>
       <c r="D280" s="2" t="inlineStr">
         <is>
-          <t>Dia 201 de 365. Provérbios 10:4: A mão diligente enriquece. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 279 de 365. Provérbios 10:4: A mão diligente enriquece. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E280" s="2" t="inlineStr">
@@ -12512,7 +12512,7 @@
       </c>
       <c r="D281" s="2" t="inlineStr">
         <is>
-          <t>Dia 202 de 365. Eclesiastes 3:1: Tudo tem o seu tempo. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 280 de 365. Eclesiastes 3:1: Tudo tem o seu tempo. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E281" s="2" t="inlineStr">
@@ -12555,7 +12555,7 @@
       </c>
       <c r="D282" s="2" t="inlineStr">
         <is>
-          <t>Dia 203 de 365. 2 Tessalonicenses 3:10-13: Não vos canseis de fazer o bem. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 281 de 365. 2 Tessalonicenses 3:10-13: Não vos canseis de fazer o bem. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E282" s="2" t="inlineStr">
@@ -12598,7 +12598,7 @@
       </c>
       <c r="D283" s="2" t="inlineStr">
         <is>
-          <t>Dia 204 de 365. Isaías 64:8: Somos o barro, Tu és o oleiro. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 282 de 365. Isaías 64:8: Somos o barro, Tu és o oleiro. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E283" s="2" t="inlineStr">
@@ -12641,7 +12641,7 @@
       </c>
       <c r="D284" s="2" t="inlineStr">
         <is>
-          <t>Dia 205 de 365. Atos 20:35: Mais bem-aventurado é dar. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 283 de 365. Atos 20:35: Mais bem-aventurado é dar. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E284" s="2" t="inlineStr">
@@ -12684,7 +12684,7 @@
       </c>
       <c r="D285" s="2" t="inlineStr">
         <is>
-          <t>Dia 206 de 365. Provérbios 16:9: Você planeja, Deus dirige. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 284 de 365. Provérbios 16:9: Você planeja, Deus dirige. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E285" s="2" t="inlineStr">
@@ -12727,7 +12727,7 @@
       </c>
       <c r="D286" s="2" t="inlineStr">
         <is>
-          <t>Dia 207 de 365. Habacuque 2:2-3: Escreva a visão. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 285 de 365. Habacuque 2:2-3: Escreva a visão. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E286" s="2" t="inlineStr">
@@ -12770,7 +12770,7 @@
       </c>
       <c r="D287" s="2" t="inlineStr">
         <is>
-          <t>Dia 208 de 365. Gênesis 39:2-3: O Senhor estava com José. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 286 de 365. Gênesis 39:2-3: O Senhor estava com José. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E287" s="2" t="inlineStr">
@@ -12813,7 +12813,7 @@
       </c>
       <c r="D288" s="2" t="inlineStr">
         <is>
-          <t>Dia 209 de 365. 1 Coríntios 10:31: Para a glória de Deus. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 287 de 365. 1 Coríntios 10:31: Para a glória de Deus. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E288" s="2" t="inlineStr">
@@ -12856,7 +12856,7 @@
       </c>
       <c r="D289" s="2" t="inlineStr">
         <is>
-          <t>Dia 210 de 365. Salmos 37:5: Entrega o teu caminho. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 288 de 365. Salmos 37:5: Entrega o teu caminho. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E289" s="2" t="inlineStr">
@@ -12899,7 +12899,7 @@
       </c>
       <c r="D290" s="2" t="inlineStr">
         <is>
-          <t>Dia 211 de 365. Zacarias 4:10: Não despreze os pequenos começos. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 289 de 365. Zacarias 4:10: Não despreze os pequenos começos. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E290" s="2" t="inlineStr">
@@ -12942,7 +12942,7 @@
       </c>
       <c r="D291" s="2" t="inlineStr">
         <is>
-          <t>Dia 212 de 365. Mateus 6:33: Busque primeiro. #fe #proposito #trabalho #palavradodia</t>
+          <t>Dia 290 de 365. Mateus 6:33: Busque primeiro. #fe #proposito #trabalho #palavradodia</t>
         </is>
       </c>
       <c r="E291" s="2" t="inlineStr">
@@ -12985,7 +12985,7 @@
       </c>
       <c r="D292" s="2" t="inlineStr">
         <is>
-          <t>Dia 213 de 365. Tiago 1:5: Precisa decidir algo e não sabe o quê? #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 291 de 365. Tiago 1:5: Precisa decidir algo e não sabe o quê? #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E292" s="2" t="inlineStr">
@@ -13028,7 +13028,7 @@
       </c>
       <c r="D293" s="2" t="inlineStr">
         <is>
-          <t>Dia 214 de 365. Provérbios 3:5-6: Não se apoie só no seu entendimento. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 292 de 365. Provérbios 3:5-6: Não se apoie só no seu entendimento. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E293" s="2" t="inlineStr">
@@ -13071,7 +13071,7 @@
       </c>
       <c r="D294" s="2" t="inlineStr">
         <is>
-          <t>Dia 215 de 365. Salmos 119:105: Uma lâmpada para os pés. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 293 de 365. Salmos 119:105: Uma lâmpada para os pés. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E294" s="2" t="inlineStr">
@@ -13114,7 +13114,7 @@
       </c>
       <c r="D295" s="2" t="inlineStr">
         <is>
-          <t>Dia 216 de 365. Provérbios 1:7: Onde a sabedoria começa. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 294 de 365. Provérbios 1:7: Onde a sabedoria começa. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E295" s="2" t="inlineStr">
@@ -13157,7 +13157,7 @@
       </c>
       <c r="D296" s="2" t="inlineStr">
         <is>
-          <t>Dia 217 de 365. Provérbios 11:14: Na multidão de conselheiros há segurança. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 295 de 365. Provérbios 11:14: Na multidão de conselheiros há segurança. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E296" s="2" t="inlineStr">
@@ -13200,7 +13200,7 @@
       </c>
       <c r="D297" s="2" t="inlineStr">
         <is>
-          <t>Dia 218 de 365. Salmos 32:8: Eu te instruirei. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 296 de 365. Salmos 32:8: Eu te instruirei. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E297" s="2" t="inlineStr">
@@ -13243,7 +13243,7 @@
       </c>
       <c r="D298" s="2" t="inlineStr">
         <is>
-          <t>Dia 219 de 365. Provérbios 4:23: Guarde o coração. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 297 de 365. Provérbios 4:23: Guarde o coração. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E298" s="2" t="inlineStr">
@@ -13286,7 +13286,7 @@
       </c>
       <c r="D299" s="2" t="inlineStr">
         <is>
-          <t>Dia 220 de 365. Isaías 30:21: Este é o caminho, andai nele. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 298 de 365. Isaías 30:21: Este é o caminho, andai nele. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E299" s="2" t="inlineStr">
@@ -13329,7 +13329,7 @@
       </c>
       <c r="D300" s="2" t="inlineStr">
         <is>
-          <t>Dia 221 de 365. Provérbios 2:6: O Senhor dá a sabedoria. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 299 de 365. Provérbios 2:6: O Senhor dá a sabedoria. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E300" s="2" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="D301" s="2" t="inlineStr">
         <is>
-          <t>Dia 222 de 365. Tiago 3:17: Como reconhecer a sabedoria que vem do alto. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 300 de 365. Tiago 3:17: Como reconhecer a sabedoria que vem do alto. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E301" s="2" t="inlineStr">
@@ -13415,7 +13415,7 @@
       </c>
       <c r="D302" s="2" t="inlineStr">
         <is>
-          <t>Dia 223 de 365. Provérbios 15:22: Sem conselho, os planos falham. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 301 de 365. Provérbios 15:22: Sem conselho, os planos falham. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E302" s="2" t="inlineStr">
@@ -13458,7 +13458,7 @@
       </c>
       <c r="D303" s="2" t="inlineStr">
         <is>
-          <t>Dia 224 de 365. Salmos 25:4-5: Mostra-me os teus caminhos. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 302 de 365. Salmos 25:4-5: Mostra-me os teus caminhos. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E303" s="2" t="inlineStr">
@@ -13501,7 +13501,7 @@
       </c>
       <c r="D304" s="2" t="inlineStr">
         <is>
-          <t>Dia 225 de 365. Provérbios 16:16: Melhor que ouro. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 303 de 365. Provérbios 16:16: Melhor que ouro. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E304" s="2" t="inlineStr">
@@ -13544,7 +13544,7 @@
       </c>
       <c r="D305" s="2" t="inlineStr">
         <is>
-          <t>Dia 226 de 365. Colossenses 3:16: Que a Palavra habite em você ricamente. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 304 de 365. Colossenses 3:16: Que a Palavra habite em você ricamente. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E305" s="2" t="inlineStr">
@@ -13587,7 +13587,7 @@
       </c>
       <c r="D306" s="2" t="inlineStr">
         <is>
-          <t>Dia 227 de 365. Provérbios 14:12: Há caminho que parece direito. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 305 de 365. Provérbios 14:12: Há caminho que parece direito. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E306" s="2" t="inlineStr">
@@ -13630,7 +13630,7 @@
       </c>
       <c r="D307" s="2" t="inlineStr">
         <is>
-          <t>Dia 228 de 365. 1 Reis 3:9: O pedido de Salomão. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 306 de 365. 1 Reis 3:9: O pedido de Salomão. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E307" s="2" t="inlineStr">
@@ -13673,7 +13673,7 @@
       </c>
       <c r="D308" s="2" t="inlineStr">
         <is>
-          <t>Dia 229 de 365. Provérbios 19:21: Muitos planos, um propósito. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 307 de 365. Provérbios 19:21: Muitos planos, um propósito. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E308" s="2" t="inlineStr">
@@ -13716,7 +13716,7 @@
       </c>
       <c r="D309" s="2" t="inlineStr">
         <is>
-          <t>Dia 230 de 365. Romanos 12:2: Não se conforme com este mundo. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 308 de 365. Romanos 12:2: Não se conforme com este mundo. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E309" s="2" t="inlineStr">
@@ -13759,7 +13759,7 @@
       </c>
       <c r="D310" s="2" t="inlineStr">
         <is>
-          <t>Dia 231 de 365. Salmos 1:1-3: Feliz quem não segue o conselho dos ímpios. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 309 de 365. Salmos 1:1-3: Feliz quem não segue o conselho dos ímpios. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E310" s="2" t="inlineStr">
@@ -13802,7 +13802,7 @@
       </c>
       <c r="D311" s="2" t="inlineStr">
         <is>
-          <t>Dia 232 de 365. Provérbios 13:20: Ande com os sábios. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 310 de 365. Provérbios 13:20: Ande com os sábios. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E311" s="2" t="inlineStr">
@@ -13845,7 +13845,7 @@
       </c>
       <c r="D312" s="2" t="inlineStr">
         <is>
-          <t>Dia 233 de 365. Eclesiastes 7:8: Melhor é o fim do que o começo. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 311 de 365. Eclesiastes 7:8: Melhor é o fim do que o começo. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E312" s="2" t="inlineStr">
@@ -13888,7 +13888,7 @@
       </c>
       <c r="D313" s="2" t="inlineStr">
         <is>
-          <t>Dia 234 de 365. Provérbios 12:15: O tolo acha que está sempre certo. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 312 de 365. Provérbios 12:15: O tolo acha que está sempre certo. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E313" s="2" t="inlineStr">
@@ -13931,7 +13931,7 @@
       </c>
       <c r="D314" s="2" t="inlineStr">
         <is>
-          <t>Dia 235 de 365. Salmos 37:23: O Senhor firma os passos do homem bom. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 313 de 365. Salmos 37:23: O Senhor firma os passos do homem bom. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E314" s="2" t="inlineStr">
@@ -13974,7 +13974,7 @@
       </c>
       <c r="D315" s="2" t="inlineStr">
         <is>
-          <t>Dia 236 de 365. Provérbios 21:5: Os planos do diligente levam à fartura. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 314 de 365. Provérbios 21:5: Os planos do diligente levam à fartura. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E315" s="2" t="inlineStr">
@@ -14017,7 +14017,7 @@
       </c>
       <c r="D316" s="2" t="inlineStr">
         <is>
-          <t>Dia 237 de 365. Filipenses 1:9-10: Discernir o que é excelente. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 315 de 365. Filipenses 1:9-10: Discernir o que é excelente. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E316" s="2" t="inlineStr">
@@ -14060,7 +14060,7 @@
       </c>
       <c r="D317" s="2" t="inlineStr">
         <is>
-          <t>Dia 238 de 365. Provérbios 18:13: Responder antes de ouvir é tolice. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 316 de 365. Provérbios 18:13: Responder antes de ouvir é tolice. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E317" s="2" t="inlineStr">
@@ -14103,7 +14103,7 @@
       </c>
       <c r="D318" s="2" t="inlineStr">
         <is>
-          <t>Dia 239 de 365. Mateus 7:24-25: Construa sobre a rocha. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 317 de 365. Mateus 7:24-25: Construa sobre a rocha. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E318" s="2" t="inlineStr">
@@ -14146,7 +14146,7 @@
       </c>
       <c r="D319" s="2" t="inlineStr">
         <is>
-          <t>Dia 240 de 365. Salmos 111:10: O temor do Senhor é o princípio da sabedoria. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 318 de 365. Salmos 111:10: O temor do Senhor é o princípio da sabedoria. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E319" s="2" t="inlineStr">
@@ -14189,7 +14189,7 @@
       </c>
       <c r="D320" s="2" t="inlineStr">
         <is>
-          <t>Dia 241 de 365. Provérbios 27:12: O prudente vê o perigo e se esconde. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 319 de 365. Provérbios 27:12: O prudente vê o perigo e se esconde. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E320" s="2" t="inlineStr">
@@ -14232,7 +14232,7 @@
       </c>
       <c r="D321" s="2" t="inlineStr">
         <is>
-          <t>Dia 242 de 365. Eclesiastes 12:13: A conclusão de tudo. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 320 de 365. Eclesiastes 12:13: A conclusão de tudo. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E321" s="2" t="inlineStr">
@@ -14275,7 +14275,7 @@
       </c>
       <c r="D322" s="2" t="inlineStr">
         <is>
-          <t>Dia 243 de 365. Daniel 2:20-21: Ele dá sabedoria aos sábios. #fe #sabedoria #decisoes #palavradodia</t>
+          <t>Dia 321 de 365. Daniel 2:20-21: Ele dá sabedoria aos sábios. #fe #sabedoria #decisoes #palavradodia</t>
         </is>
       </c>
       <c r="E322" s="2" t="inlineStr">
@@ -14318,7 +14318,7 @@
       </c>
       <c r="D323" s="2" t="inlineStr">
         <is>
-          <t>Dia 244 de 365. Filipenses 4:13: Tudo posso naquele que me fortalece. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 322 de 365. Filipenses 4:13: Tudo posso naquele que me fortalece. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E323" s="2" t="inlineStr">
@@ -14361,7 +14361,7 @@
       </c>
       <c r="D324" s="2" t="inlineStr">
         <is>
-          <t>Dia 245 de 365. Hebreus 12:1-2: Corra com perseverança. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 323 de 365. Hebreus 12:1-2: Corra com perseverança. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E324" s="2" t="inlineStr">
@@ -14404,7 +14404,7 @@
       </c>
       <c r="D325" s="2" t="inlineStr">
         <is>
-          <t>Dia 246 de 365. Salmos 27:13: Eu creio que verei a bondade do Senhor. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 324 de 365. Salmos 27:13: Eu creio que verei a bondade do Senhor. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E325" s="2" t="inlineStr">
@@ -14447,7 +14447,7 @@
       </c>
       <c r="D326" s="2" t="inlineStr">
         <is>
-          <t>Dia 247 de 365. Tiago 1:2-4: Alegria nas provações? #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 325 de 365. Tiago 1:2-4: Alegria nas provações? #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E326" s="2" t="inlineStr">
@@ -14490,7 +14490,7 @@
       </c>
       <c r="D327" s="2" t="inlineStr">
         <is>
-          <t>Dia 248 de 365. Provérbios 24:16: O justo cai sete vezes e se levanta. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 326 de 365. Provérbios 24:16: O justo cai sete vezes e se levanta. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E327" s="2" t="inlineStr">
@@ -14533,7 +14533,7 @@
       </c>
       <c r="D328" s="2" t="inlineStr">
         <is>
-          <t>Dia 249 de 365. 2 Timóteo 4:7: Combati o bom combate. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 327 de 365. 2 Timóteo 4:7: Combati o bom combate. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E328" s="2" t="inlineStr">
@@ -14576,7 +14576,7 @@
       </c>
       <c r="D329" s="2" t="inlineStr">
         <is>
-          <t>Dia 250 de 365. Salmos 18:32: Deus me reveste de força. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 328 de 365. Salmos 18:32: Deus me reveste de força. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E329" s="2" t="inlineStr">
@@ -14619,7 +14619,7 @@
       </c>
       <c r="D330" s="2" t="inlineStr">
         <is>
-          <t>Dia 251 de 365. Salmos 66:10-12: Passamos pelo fogo e pela água. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 329 de 365. Salmos 66:10-12: Passamos pelo fogo e pela água. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E330" s="2" t="inlineStr">
@@ -14662,7 +14662,7 @@
       </c>
       <c r="D331" s="2" t="inlineStr">
         <is>
-          <t>Dia 252 de 365. Salmos 73:26: Quando o corpo e o coração falham. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 330 de 365. Salmos 73:26: Quando o corpo e o coração falham. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E331" s="2" t="inlineStr">
@@ -14705,7 +14705,7 @@
       </c>
       <c r="D332" s="2" t="inlineStr">
         <is>
-          <t>Dia 253 de 365. Isaías 41:13: Eu te ajudo. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 331 de 365. Isaías 41:13: Eu te ajudo. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E332" s="2" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="D333" s="2" t="inlineStr">
         <is>
-          <t>Dia 254 de 365. 1 Coríntios 16:13: Sede fortes. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 332 de 365. 1 Coríntios 16:13: Sede fortes. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E333" s="2" t="inlineStr">
@@ -14791,7 +14791,7 @@
       </c>
       <c r="D334" s="2" t="inlineStr">
         <is>
-          <t>Dia 255 de 365. Efésios 6:10: Fortalecei-vos no Senhor. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 333 de 365. Efésios 6:10: Fortalecei-vos no Senhor. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E334" s="2" t="inlineStr">
@@ -14834,7 +14834,7 @@
       </c>
       <c r="D335" s="2" t="inlineStr">
         <is>
-          <t>Dia 256 de 365. Salmos 28:7: O Senhor é a minha força e o meu escudo. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 334 de 365. Salmos 28:7: O Senhor é a minha força e o meu escudo. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E335" s="2" t="inlineStr">
@@ -14877,7 +14877,7 @@
       </c>
       <c r="D336" s="2" t="inlineStr">
         <is>
-          <t>Dia 257 de 365. Hebreus 10:36: Vocês precisam de perseverança. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 335 de 365. Hebreus 10:36: Vocês precisam de perseverança. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E336" s="2" t="inlineStr">
@@ -14920,7 +14920,7 @@
       </c>
       <c r="D337" s="2" t="inlineStr">
         <is>
-          <t>Dia 258 de 365. Zacarias 4:6: Não por força, nem por violência. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 336 de 365. Zacarias 4:6: Não por força, nem por violência. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E337" s="2" t="inlineStr">
@@ -14963,7 +14963,7 @@
       </c>
       <c r="D338" s="2" t="inlineStr">
         <is>
-          <t>Dia 259 de 365. Isaías 50:7: Pus o meu rosto como pedra. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 337 de 365. Isaías 50:7: Pus o meu rosto como pedra. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E338" s="2" t="inlineStr">
@@ -15006,7 +15006,7 @@
       </c>
       <c r="D339" s="2" t="inlineStr">
         <is>
-          <t>Dia 260 de 365. Salmos 138:7: Ainda que eu ande no meio da angústia. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 338 de 365. Salmos 138:7: Ainda que eu ande no meio da angústia. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E339" s="2" t="inlineStr">
@@ -15049,7 +15049,7 @@
       </c>
       <c r="D340" s="2" t="inlineStr">
         <is>
-          <t>Dia 261 de 365. Neemias 6:3: Estou fazendo uma grande obra. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 339 de 365. Neemias 6:3: Estou fazendo uma grande obra. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E340" s="2" t="inlineStr">
@@ -15092,7 +15092,7 @@
       </c>
       <c r="D341" s="2" t="inlineStr">
         <is>
-          <t>Dia 262 de 365. Tiago 1:12: Feliz o que suporta a provação. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 340 de 365. Tiago 1:12: Feliz o que suporta a provação. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E341" s="2" t="inlineStr">
@@ -15135,7 +15135,7 @@
       </c>
       <c r="D342" s="2" t="inlineStr">
         <is>
-          <t>Dia 263 de 365. Salmos 46:5: Deus está no meio dela. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 341 de 365. Salmos 46:5: Deus está no meio dela. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E342" s="2" t="inlineStr">
@@ -15178,7 +15178,7 @@
       </c>
       <c r="D343" s="2" t="inlineStr">
         <is>
-          <t>Dia 264 de 365. Hebreus 12:11: A disciplina dói, depois dá fruto. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 342 de 365. Hebreus 12:11: A disciplina dói, depois dá fruto. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E343" s="2" t="inlineStr">
@@ -15221,7 +15221,7 @@
       </c>
       <c r="D344" s="2" t="inlineStr">
         <is>
-          <t>Dia 265 de 365. Lucas 18:1: Orar sempre e nunca desistir. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 343 de 365. Lucas 18:1: Orar sempre e nunca desistir. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E344" s="2" t="inlineStr">
@@ -15264,7 +15264,7 @@
       </c>
       <c r="D345" s="2" t="inlineStr">
         <is>
-          <t>Dia 266 de 365. Salmos 37:24: Ainda que caia, não ficará prostrado. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 344 de 365. Salmos 37:24: Ainda que caia, não ficará prostrado. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E345" s="2" t="inlineStr">
@@ -15307,7 +15307,7 @@
       </c>
       <c r="D346" s="2" t="inlineStr">
         <is>
-          <t>Dia 267 de 365. 2 Coríntios 4:7: Um tesouro em vasos de barro. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 345 de 365. 2 Coríntios 4:7: Um tesouro em vasos de barro. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E346" s="2" t="inlineStr">
@@ -15350,7 +15350,7 @@
       </c>
       <c r="D347" s="2" t="inlineStr">
         <is>
-          <t>Dia 268 de 365. Josué 14:11: Calebe com 85 anos. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 346 de 365. Josué 14:11: Calebe com 85 anos. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E347" s="2" t="inlineStr">
@@ -15393,7 +15393,7 @@
       </c>
       <c r="D348" s="2" t="inlineStr">
         <is>
-          <t>Dia 269 de 365. Isaías 40:28: Deus não se cansa. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 347 de 365. Isaías 40:28: Deus não se cansa. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E348" s="2" t="inlineStr">
@@ -15436,7 +15436,7 @@
       </c>
       <c r="D349" s="2" t="inlineStr">
         <is>
-          <t>Dia 270 de 365. Romanos 8:37: Mais que vencedores. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 348 de 365. Romanos 8:37: Mais que vencedores. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E349" s="2" t="inlineStr">
@@ -15479,7 +15479,7 @@
       </c>
       <c r="D350" s="2" t="inlineStr">
         <is>
-          <t>Dia 271 de 365. Habacuque 3:19: Pés como os das corças. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 349 de 365. Habacuque 3:19: Pés como os das corças. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E350" s="2" t="inlineStr">
@@ -15522,7 +15522,7 @@
       </c>
       <c r="D351" s="2" t="inlineStr">
         <is>
-          <t>Dia 272 de 365. Apocalipse 2:10: Sê fiel até a morte. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 350 de 365. Apocalipse 2:10: Sê fiel até a morte. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E351" s="2" t="inlineStr">
@@ -15565,7 +15565,7 @@
       </c>
       <c r="D352" s="2" t="inlineStr">
         <is>
-          <t>Dia 273 de 365. 2 Crônicas 15:7: Não desfaleçam as vossas mãos. #fe #perseveranca #forca #palavradodia</t>
+          <t>Dia 351 de 365. 2 Crônicas 15:7: Não desfaleçam as vossas mãos. #fe #perseveranca #forca #palavradodia</t>
         </is>
       </c>
       <c r="E352" s="2" t="inlineStr">
@@ -15608,7 +15608,7 @@
       </c>
       <c r="D353" s="2" t="inlineStr">
         <is>
-          <t>Dia 274 de 365. João 3:16: O versículo mais conhecido da Bíblia. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 352 de 365. João 3:16: O versículo mais conhecido da Bíblia. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E353" s="2" t="inlineStr">
@@ -15651,7 +15651,7 @@
       </c>
       <c r="D354" s="2" t="inlineStr">
         <is>
-          <t>Dia 275 de 365. 1 João 4:8: Deus é amor. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 353 de 365. 1 João 4:8: Deus é amor. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E354" s="2" t="inlineStr">
@@ -15694,7 +15694,7 @@
       </c>
       <c r="D355" s="2" t="inlineStr">
         <is>
-          <t>Dia 276 de 365. Romanos 5:8: Ele te amou no seu pior momento. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 354 de 365. Romanos 5:8: Ele te amou no seu pior momento. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E355" s="2" t="inlineStr">
@@ -15737,7 +15737,7 @@
       </c>
       <c r="D356" s="2" t="inlineStr">
         <is>
-          <t>Dia 277 de 365. Romanos 8:38-39: Nada pode te separar. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 355 de 365. Romanos 8:38-39: Nada pode te separar. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E356" s="2" t="inlineStr">
@@ -15780,7 +15780,7 @@
       </c>
       <c r="D357" s="2" t="inlineStr">
         <is>
-          <t>Dia 278 de 365. 1 João 4:19: Nós amamos porque Ele nos amou primeiro. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 356 de 365. 1 João 4:19: Nós amamos porque Ele nos amou primeiro. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E357" s="2" t="inlineStr">
@@ -15823,7 +15823,7 @@
       </c>
       <c r="D358" s="2" t="inlineStr">
         <is>
-          <t>Dia 279 de 365. Jeremias 31:3: Com amor eterno eu te amei. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 357 de 365. Jeremias 31:3: Com amor eterno eu te amei. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E358" s="2" t="inlineStr">
@@ -15866,7 +15866,7 @@
       </c>
       <c r="D359" s="2" t="inlineStr">
         <is>
-          <t>Dia 280 de 365. 1 Coríntios 13:7: Tudo sofre, tudo crê, tudo espera, tudo suporta. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 358 de 365. 1 Coríntios 13:7: Tudo sofre, tudo crê, tudo espera, tudo suporta. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E359" s="2" t="inlineStr">
@@ -15909,7 +15909,7 @@
       </c>
       <c r="D360" s="2" t="inlineStr">
         <is>
-          <t>Dia 281 de 365. 1 Coríntios 13:13: O maior deles é o amor. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 359 de 365. 1 Coríntios 13:13: O maior deles é o amor. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E360" s="2" t="inlineStr">
@@ -15952,7 +15952,7 @@
       </c>
       <c r="D361" s="2" t="inlineStr">
         <is>
-          <t>Dia 282 de 365. Mateus 22:37-39: Os dois maiores mandamentos. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 360 de 365. Mateus 22:37-39: Os dois maiores mandamentos. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E361" s="2" t="inlineStr">
@@ -15995,7 +15995,7 @@
       </c>
       <c r="D362" s="2" t="inlineStr">
         <is>
-          <t>Dia 283 de 365. João 13:34-35: Um mandamento novo. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 361 de 365. João 13:34-35: Um mandamento novo. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E362" s="2" t="inlineStr">
@@ -16038,7 +16038,7 @@
       </c>
       <c r="D363" s="2" t="inlineStr">
         <is>
-          <t>Dia 284 de 365. Lucas 6:27-28: Amai os vossos inimigos. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 362 de 365. Lucas 6:27-28: Amai os vossos inimigos. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E363" s="2" t="inlineStr">
@@ -16081,7 +16081,7 @@
       </c>
       <c r="D364" s="2" t="inlineStr">
         <is>
-          <t>Dia 285 de 365. Efésios 3:17-19: Largura, comprimento, altura e profundidade. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 363 de 365. Efésios 3:17-19: Largura, comprimento, altura e profundidade. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E364" s="2" t="inlineStr">
@@ -16124,7 +16124,7 @@
       </c>
       <c r="D365" s="2" t="inlineStr">
         <is>
-          <t>Dia 286 de 365. 1 João 3:18: Amor de verdade aparece em ações. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 364 de 365. 1 João 3:18: Amor de verdade aparece em ações. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E365" s="2" t="inlineStr">
@@ -16167,7 +16167,7 @@
       </c>
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>Dia 287 de 365. Romanos 13:10: O amor não faz mal ao próximo. #fe #amordedeus #amor #palavradodia</t>
+          <t>Dia 365 de 365. Romanos 13:10: O amor não faz mal ao próximo. #fe #amordedeus #amor #palavradodia</t>
         </is>
       </c>
       <c r="E366" s="2" t="inlineStr">

</xml_diff>